<commit_message>
Update service resource model to reflect accurate infrastructure details
Update the SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx file to reflect the corrected infrastructure details, specifically noting single FortiGate instance and VPCs instead of VPS.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 2280164f-bb82-4478-b7ec-31748819b312
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
+++ b/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
@@ -5924,46 +5924,46 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A4:AL18"/>
+  <dimension ref="A4:AL19"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="24.83203125" customWidth="1"/>
-    <col min="11" max="11" width="24.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="24.83203125" customWidth="1"/>
-    <col min="17" max="17" width="24.83203125" customWidth="1"/>
-    <col min="18" max="18" width="24.83203125" customWidth="1"/>
-    <col min="19" max="19" width="24.83203125" customWidth="1"/>
-    <col min="20" max="20" width="24.83203125" customWidth="1"/>
-    <col min="21" max="21" width="24.83203125" customWidth="1"/>
-    <col min="22" max="22" width="24.83203125" customWidth="1"/>
-    <col min="23" max="23" width="24.83203125" customWidth="1"/>
-    <col min="24" max="24" width="24.83203125" customWidth="1"/>
-    <col min="25" max="25" width="24.83203125" customWidth="1"/>
-    <col min="26" max="26" width="24.83203125" customWidth="1"/>
-    <col min="27" max="27" width="24.83203125" customWidth="1"/>
-    <col min="28" max="28" width="24.83203125" customWidth="1"/>
-    <col min="29" max="29" width="24.83203125" customWidth="1"/>
-    <col min="30" max="30" width="24.83203125" customWidth="1"/>
-    <col min="31" max="31" width="24.83203125" customWidth="1"/>
-    <col min="32" max="32" width="24.83203125" customWidth="1"/>
-    <col min="33" max="33" width="24.83203125" customWidth="1"/>
-    <col min="34" max="34" width="24.83203125" customWidth="1"/>
-    <col min="35" max="35" width="24.83203125" customWidth="1"/>
-    <col min="36" max="36" width="24.83203125" customWidth="1"/>
-    <col min="37" max="37" width="24.83203125" customWidth="1"/>
-    <col min="38" max="38" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+    <col min="9" max="9" width="26.83203125" customWidth="1"/>
+    <col min="10" max="10" width="26.83203125" customWidth="1"/>
+    <col min="11" max="11" width="26.83203125" customWidth="1"/>
+    <col min="12" max="12" width="26.83203125" customWidth="1"/>
+    <col min="13" max="13" width="26.83203125" customWidth="1"/>
+    <col min="14" max="14" width="26.83203125" customWidth="1"/>
+    <col min="15" max="15" width="26.83203125" customWidth="1"/>
+    <col min="16" max="16" width="26.83203125" customWidth="1"/>
+    <col min="17" max="17" width="26.83203125" customWidth="1"/>
+    <col min="18" max="18" width="26.83203125" customWidth="1"/>
+    <col min="19" max="19" width="26.83203125" customWidth="1"/>
+    <col min="20" max="20" width="26.83203125" customWidth="1"/>
+    <col min="21" max="21" width="26.83203125" customWidth="1"/>
+    <col min="22" max="22" width="26.83203125" customWidth="1"/>
+    <col min="23" max="23" width="26.83203125" customWidth="1"/>
+    <col min="24" max="24" width="26.83203125" customWidth="1"/>
+    <col min="25" max="25" width="26.83203125" customWidth="1"/>
+    <col min="26" max="26" width="26.83203125" customWidth="1"/>
+    <col min="27" max="27" width="26.83203125" customWidth="1"/>
+    <col min="28" max="28" width="26.83203125" customWidth="1"/>
+    <col min="29" max="29" width="26.83203125" customWidth="1"/>
+    <col min="30" max="30" width="26.83203125" customWidth="1"/>
+    <col min="31" max="31" width="26.83203125" customWidth="1"/>
+    <col min="32" max="32" width="26.83203125" customWidth="1"/>
+    <col min="33" max="33" width="26.83203125" customWidth="1"/>
+    <col min="34" max="34" width="26.83203125" customWidth="1"/>
+    <col min="35" max="35" width="26.83203125" customWidth="1"/>
+    <col min="36" max="36" width="26.83203125" customWidth="1"/>
+    <col min="37" max="37" width="26.83203125" customWidth="1"/>
+    <col min="38" max="38" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4">
@@ -6294,7 +6294,7 @@
         <v>Multinodo Cluster</v>
       </c>
       <c r="K8" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>Seeweb Multinodo Italy (DC1)</v>
       </c>
       <c r="L8" t="str">
         <v>Resources - SW configuration</v>
@@ -6354,7 +6354,7 @@
         <v>1 week</v>
       </c>
       <c r="AE8" t="str">
-        <v xml:space="preserve">Zone Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF8" t="str">
         <v>Automated By App</v>
@@ -6369,13 +6369,13 @@
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ8" t="str">
-        <v>VM Management, Backup, Snapshot</v>
+        <v>VM Mgmt, PBS Replication</v>
       </c>
       <c r="AK8" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL8" t="str">
-        <v>Seeweb Multinodo Contract</v>
+        <v>Seeweb Multinodo + PBS</v>
       </c>
     </row>
     <row r="9">
@@ -6398,19 +6398,19 @@
         <v>Vendor Private</v>
       </c>
       <c r="G9" t="str">
-        <v>HW Appliance</v>
+        <v>Full IaaS</v>
       </c>
       <c r="H9" t="str">
-        <v>Fortinet Inc.</v>
+        <v>Proxmox Server Solutions GmbH</v>
       </c>
       <c r="I9" t="str">
-        <v>HW Appliance - FortiGate NGFW</v>
+        <v>Bare Metal-Linux OS</v>
       </c>
       <c r="J9" t="str">
-        <v>2 (HA Cluster)</v>
+        <v>1 (Dedicato)</v>
       </c>
       <c r="K9" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>Seeweb Italy (DC2 - DR Site)</v>
       </c>
       <c r="L9" t="str">
         <v>Resources - SW configuration</v>
@@ -6419,10 +6419,10 @@
         <v>Active</v>
       </c>
       <c r="N9" t="str">
-        <v>Fixed capacity</v>
+        <v>Ops Manual</v>
       </c>
       <c r="O9" t="str">
-        <v>Do not scale - Fixed capacity</v>
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P9" t="str">
         <v>No outages</v>
@@ -6440,13 +6440,13 @@
         <v>File (TXT)</v>
       </c>
       <c r="U9" t="str">
-        <v>7.4.x</v>
+        <v>3.x</v>
       </c>
       <c r="V9" t="str">
         <v>SW Bins</v>
       </c>
       <c r="W9" t="str">
-        <v>Private Others Registry</v>
+        <v>Object Store (SW bins)</v>
       </c>
       <c r="X9" t="str">
         <v>Resource Recovery</v>
@@ -6464,13 +6464,13 @@
         <v>1 month</v>
       </c>
       <c r="AC9" t="str">
-        <v>N/A</v>
+        <v>1 min</v>
       </c>
       <c r="AD9" t="str">
-        <v>N/A</v>
+        <v>1 week</v>
       </c>
       <c r="AE9" t="str">
-        <v xml:space="preserve">Local Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF9" t="str">
         <v>Manual By Operation</v>
@@ -6479,19 +6479,19 @@
         <v>Hour (1-5)</v>
       </c>
       <c r="AH9" t="str">
-        <v>Hour (1-5)</v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AI9" t="str">
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ9" t="str">
-        <v>Security, Threat Monitoring</v>
+        <v>Backup Storage, DR</v>
       </c>
       <c r="AK9" t="str">
-        <v>COTs SW License</v>
+        <v>Public Cloud Consumption</v>
       </c>
       <c r="AL9" t="str">
-        <v>FortiCare + FortiGuard</v>
+        <v>Seeweb PBS Dedicated</v>
       </c>
     </row>
     <row r="10">
@@ -6499,10 +6499,10 @@
         <v>PROD</v>
       </c>
       <c r="B10" t="str">
-        <v>99,9%</v>
+        <v>99,5%</v>
       </c>
       <c r="C10" t="str">
-        <v>HA</v>
+        <v>HA-</v>
       </c>
       <c r="D10" t="str">
         <v>CORE PLATFORM</v>
@@ -6514,19 +6514,19 @@
         <v>Vendor Private</v>
       </c>
       <c r="G10" t="str">
-        <v>Full IaaS</v>
+        <v>HW Appliance</v>
       </c>
       <c r="H10" t="str">
-        <v>W3Suite (Easy Digital Group)</v>
+        <v>Fortinet Inc.</v>
       </c>
       <c r="I10" t="str">
-        <v>App (RunTime) - Linux native</v>
+        <v>HW Appliance - FortiGate NGFW</v>
       </c>
       <c r="J10" t="str">
-        <v>3 VPS dedicate</v>
+        <v>1 (Single)</v>
       </c>
       <c r="K10" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>Seeweb Multinodo Italy (DC1)</v>
       </c>
       <c r="L10" t="str">
         <v>Resources - SW configuration</v>
@@ -6535,16 +6535,16 @@
         <v>Active</v>
       </c>
       <c r="N10" t="str">
-        <v>Ops Manual</v>
+        <v>Fixed capacity</v>
       </c>
       <c r="O10" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+        <v>Do not scale - Fixed capacity</v>
       </c>
       <c r="P10" t="str">
         <v>No outages</v>
       </c>
       <c r="Q10" t="str">
-        <v>Ops - Automated</v>
+        <v>Ops - Manual</v>
       </c>
       <c r="R10" t="str">
         <v>Ops Manual - direct Log-on resource</v>
@@ -6553,16 +6553,16 @@
         <v>No outages</v>
       </c>
       <c r="T10" t="str">
-        <v>File (Ansible playbook) - VM configuration</v>
+        <v>File (TXT)</v>
       </c>
       <c r="U10" t="str">
-        <v>SemVer</v>
+        <v>7.4.x</v>
       </c>
       <c r="V10" t="str">
         <v>SW Bins</v>
       </c>
       <c r="W10" t="str">
-        <v>Object Store (SW bins)</v>
+        <v>Private Others Registry</v>
       </c>
       <c r="X10" t="str">
         <v>Resource Recovery</v>
@@ -6580,34 +6580,34 @@
         <v>1 month</v>
       </c>
       <c r="AC10" t="str">
-        <v>1 min</v>
+        <v>N/A</v>
       </c>
       <c r="AD10" t="str">
-        <v>1 week</v>
+        <v>N/A</v>
       </c>
       <c r="AE10" t="str">
-        <v xml:space="preserve">Zone Resilent </v>
+        <v xml:space="preserve">Local Resilent </v>
       </c>
       <c r="AF10" t="str">
-        <v>Automated By App</v>
+        <v>Manual By Operation</v>
       </c>
       <c r="AG10" t="str">
-        <v>Minutes (1-5)</v>
+        <v>Hour (1-5)</v>
       </c>
       <c r="AH10" t="str">
-        <v xml:space="preserve">Seconds </v>
+        <v>Hour (1-5)</v>
       </c>
       <c r="AI10" t="str">
-        <v>SW Integrator</v>
+        <v>HW/SW vendor</v>
       </c>
       <c r="AJ10" t="str">
-        <v>Deploy, Monitoring</v>
+        <v>Security, Monitoring</v>
       </c>
       <c r="AK10" t="str">
-        <v>Public Cloud Consumption</v>
+        <v>COTs SW License</v>
       </c>
       <c r="AL10" t="str">
-        <v>Seeweb VPS + W3Suite License</v>
+        <v>FortiCare + FortiGuard</v>
       </c>
     </row>
     <row r="11">
@@ -6633,16 +6633,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H11" t="str">
-        <v>F5 Networks (Nginx)</v>
+        <v>W3Suite (Easy Digital Group)</v>
       </c>
       <c r="I11" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J11" t="str">
-        <v>2 VPS dedicate</v>
+        <v>3 VPC</v>
       </c>
       <c r="K11" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>Seeweb Multinodo Italy (DC1)</v>
       </c>
       <c r="L11" t="str">
         <v>Resources - SW configuration</v>
@@ -6660,7 +6660,7 @@
         <v>No outages</v>
       </c>
       <c r="Q11" t="str">
-        <v>Ops - Manual</v>
+        <v>Ops - Automated</v>
       </c>
       <c r="R11" t="str">
         <v>Ops Manual - direct Log-on resource</v>
@@ -6669,10 +6669,10 @@
         <v>No outages</v>
       </c>
       <c r="T11" t="str">
-        <v>File (TXT)</v>
+        <v>File (Ansible playbook) - VM configuration</v>
       </c>
       <c r="U11" t="str">
-        <v>1.24.x</v>
+        <v>SemVer</v>
       </c>
       <c r="V11" t="str">
         <v>SW Bins</v>
@@ -6696,34 +6696,34 @@
         <v>1 month</v>
       </c>
       <c r="AC11" t="str">
-        <v>N/A</v>
+        <v>1 min</v>
       </c>
       <c r="AD11" t="str">
-        <v>N/A</v>
+        <v>1 week</v>
       </c>
       <c r="AE11" t="str">
-        <v xml:space="preserve">Local Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF11" t="str">
         <v>Automated By App</v>
       </c>
       <c r="AG11" t="str">
+        <v>Minutes (1-5)</v>
+      </c>
+      <c r="AH11" t="str">
         <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AH11" t="str">
-        <v>N/A</v>
       </c>
       <c r="AI11" t="str">
         <v>SW Integrator</v>
       </c>
       <c r="AJ11" t="str">
-        <v>TLS, Config</v>
+        <v>Deploy, Monitoring</v>
       </c>
       <c r="AK11" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL11" t="str">
-        <v>Seeweb VPS</v>
+        <v>Seeweb VPC + W3Suite</v>
       </c>
     </row>
     <row r="12">
@@ -6749,16 +6749,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H12" t="str">
-        <v>Redis Ltd</v>
+        <v>F5 Networks (Nginx)</v>
       </c>
       <c r="I12" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J12" t="str">
-        <v>2 VPS dedicate</v>
+        <v>2 VPC</v>
       </c>
       <c r="K12" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>Seeweb Multinodo Italy (DC1)</v>
       </c>
       <c r="L12" t="str">
         <v>Resources - SW configuration</v>
@@ -6788,7 +6788,7 @@
         <v>File (TXT)</v>
       </c>
       <c r="U12" t="str">
-        <v>7.2.x</v>
+        <v>1.24.x</v>
       </c>
       <c r="V12" t="str">
         <v>SW Bins</v>
@@ -6812,13 +6812,13 @@
         <v>1 month</v>
       </c>
       <c r="AC12" t="str">
-        <v>1 min</v>
+        <v>N/A</v>
       </c>
       <c r="AD12" t="str">
-        <v>1 week</v>
+        <v>N/A</v>
       </c>
       <c r="AE12" t="str">
-        <v xml:space="preserve">Local Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF12" t="str">
         <v>Automated By App</v>
@@ -6827,19 +6827,19 @@
         <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AH12" t="str">
-        <v xml:space="preserve">Seconds </v>
+        <v>N/A</v>
       </c>
       <c r="AI12" t="str">
         <v>SW Integrator</v>
       </c>
       <c r="AJ12" t="str">
-        <v>Memory Monitoring</v>
+        <v>TLS, Config</v>
       </c>
       <c r="AK12" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL12" t="str">
-        <v>Seeweb VPS</v>
+        <v>Seeweb VPC</v>
       </c>
     </row>
     <row r="13">
@@ -6853,7 +6853,7 @@
         <v>HA</v>
       </c>
       <c r="D13" t="str">
-        <v>DATABASE LAYER</v>
+        <v>CORE PLATFORM</v>
       </c>
       <c r="E13" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6865,16 +6865,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H13" t="str">
-        <v>PostgreSQL Global Development Group</v>
+        <v>Redis Ltd</v>
       </c>
       <c r="I13" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J13" t="str">
-        <v>2 VPS (Primary+Replica)</v>
+        <v>2 VPC</v>
       </c>
       <c r="K13" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>Seeweb Multinodo Italy (DC1)</v>
       </c>
       <c r="L13" t="str">
         <v>Resources - SW configuration</v>
@@ -6889,7 +6889,7 @@
         <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P13" t="str">
-        <v>Minutes (1-10)</v>
+        <v>No outages</v>
       </c>
       <c r="Q13" t="str">
         <v>Ops - Manual</v>
@@ -6898,13 +6898,13 @@
         <v>Ops Manual - direct Log-on resource</v>
       </c>
       <c r="S13" t="str">
-        <v>Minutes (1-10)</v>
+        <v>No outages</v>
       </c>
       <c r="T13" t="str">
         <v>File (TXT)</v>
       </c>
       <c r="U13" t="str">
-        <v>15.x</v>
+        <v>7.2.x</v>
       </c>
       <c r="V13" t="str">
         <v>SW Bins</v>
@@ -6913,7 +6913,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X13" t="str">
-        <v>Resource: Release and Recovery</v>
+        <v>Resource Recovery</v>
       </c>
       <c r="Y13" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -6934,13 +6934,13 @@
         <v>1 week</v>
       </c>
       <c r="AE13" t="str">
-        <v xml:space="preserve">Zone Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF13" t="str">
         <v>Automated By App</v>
       </c>
       <c r="AG13" t="str">
-        <v>Minutes (1-5)</v>
+        <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AH13" t="str">
         <v xml:space="preserve">Seconds </v>
@@ -6949,13 +6949,13 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ13" t="str">
-        <v>Backup, Tuning, PITR</v>
+        <v>Memory Monitoring</v>
       </c>
       <c r="AK13" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL13" t="str">
-        <v>Seeweb VPS</v>
+        <v>Seeweb VPC</v>
       </c>
     </row>
     <row r="14">
@@ -6981,16 +6981,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H14" t="str">
-        <v>Seeweb S.r.l. (Ceph Storage)</v>
+        <v>PostgreSQL Global Development Group</v>
       </c>
       <c r="I14" t="str">
-        <v>Bare Metal-Linux OS</v>
+        <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J14" t="str">
-        <v>Cluster Ceph Seeweb</v>
+        <v>2 VPC (Primary+Replica)</v>
       </c>
       <c r="K14" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>Seeweb Multinodo Italy (DC1)</v>
       </c>
       <c r="L14" t="str">
         <v>Resources - SW configuration</v>
@@ -7005,7 +7005,7 @@
         <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P14" t="str">
-        <v>No outages</v>
+        <v>Minutes (1-10)</v>
       </c>
       <c r="Q14" t="str">
         <v>Ops - Manual</v>
@@ -7014,13 +7014,13 @@
         <v>Ops Manual - direct Log-on resource</v>
       </c>
       <c r="S14" t="str">
-        <v>No outages</v>
+        <v>Minutes (1-10)</v>
       </c>
       <c r="T14" t="str">
         <v>File (TXT)</v>
       </c>
       <c r="U14" t="str">
-        <v>Quincy</v>
+        <v>15.x</v>
       </c>
       <c r="V14" t="str">
         <v>SW Bins</v>
@@ -7029,7 +7029,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X14" t="str">
-        <v>Resource Recovery</v>
+        <v>Resource: Release and Recovery</v>
       </c>
       <c r="Y14" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -7050,28 +7050,28 @@
         <v>1 week</v>
       </c>
       <c r="AE14" t="str">
-        <v xml:space="preserve">Zone Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF14" t="str">
         <v>Automated By App</v>
       </c>
       <c r="AG14" t="str">
-        <v xml:space="preserve">Seconds </v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AH14" t="str">
         <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AI14" t="str">
-        <v>HW/SW vendor</v>
+        <v>SW Integrator</v>
       </c>
       <c r="AJ14" t="str">
-        <v>Capacity, Health</v>
+        <v>Backup, Tuning, PITR</v>
       </c>
       <c r="AK14" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL14" t="str">
-        <v>Seeweb Storage</v>
+        <v>Seeweb VPC</v>
       </c>
     </row>
     <row r="15">
@@ -7079,115 +7079,115 @@
         <v>PROD</v>
       </c>
       <c r="B15" t="str">
-        <v>99,5%</v>
+        <v>99,9%</v>
       </c>
       <c r="C15" t="str">
-        <v>HA-</v>
+        <v>HA</v>
       </c>
       <c r="D15" t="str">
-        <v>AI SERVICES</v>
+        <v>DATABASE LAYER</v>
       </c>
       <c r="E15" t="str">
-        <v>Not W3 Public cloud Tenant</v>
+        <v>Not W3 Private datacenter</v>
       </c>
       <c r="F15" t="str">
         <v>Vendor Private</v>
       </c>
       <c r="G15" t="str">
-        <v>Multi-tenant SaaS</v>
+        <v>Full IaaS</v>
       </c>
       <c r="H15" t="str">
-        <v>OpenAI</v>
+        <v>Seeweb S.r.l. (Ceph Storage)</v>
       </c>
       <c r="I15" t="str">
-        <v>SaaS  App - Generic Platform</v>
+        <v>Bare Metal-Linux OS</v>
       </c>
       <c r="J15" t="str">
-        <v>SaaS</v>
+        <v>Cluster Ceph</v>
       </c>
       <c r="K15" t="str">
-        <v>OpenAI Cloud (EU)</v>
+        <v>Seeweb Multinodo Italy (DC1)</v>
       </c>
       <c r="L15" t="str">
-        <v xml:space="preserve">Internal SaaS/Cloud provider -configuration  </v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M15" t="str">
         <v>Active</v>
       </c>
       <c r="N15" t="str">
-        <v>Full Automated</v>
+        <v>Ops Manual</v>
       </c>
       <c r="O15" t="str">
-        <v>Native autoscale (SaaS /Cloud providers)</v>
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P15" t="str">
         <v>No outages</v>
       </c>
       <c r="Q15" t="str">
-        <v>Fully Automated</v>
+        <v>Ops - Manual</v>
       </c>
       <c r="R15" t="str">
-        <v>Automated By SaaS/Cloud Provider</v>
+        <v>Ops Manual - direct Log-on resource</v>
       </c>
       <c r="S15" t="str">
         <v>No outages</v>
       </c>
       <c r="T15" t="str">
-        <v>Database (metadata) - section of application data App configuration</v>
+        <v>File (TXT)</v>
       </c>
       <c r="U15" t="str">
-        <v>API v1</v>
+        <v>Quincy</v>
       </c>
       <c r="V15" t="str">
-        <v>N/A</v>
+        <v>SW Bins</v>
       </c>
       <c r="W15" t="str">
-        <v>N/A</v>
+        <v>Object Store (SW bins)</v>
       </c>
       <c r="X15" t="str">
-        <v>N/A</v>
+        <v>Resource Recovery</v>
       </c>
       <c r="Y15" t="str">
-        <v>N/A</v>
+        <v>On-Premise SW/Appliance</v>
       </c>
       <c r="Z15" t="str">
-        <v>N/A</v>
+        <v>On-premise Store (Appliance)</v>
       </c>
       <c r="AA15" t="str">
-        <v>N/A</v>
+        <v>Daily</v>
       </c>
       <c r="AB15" t="str">
-        <v>N/A</v>
+        <v>1 month</v>
       </c>
       <c r="AC15" t="str">
-        <v>N/A</v>
+        <v>1 min</v>
       </c>
       <c r="AD15" t="str">
-        <v>N/A</v>
+        <v>1 week</v>
       </c>
       <c r="AE15" t="str">
-        <v xml:space="preserve">Region Resilent </v>
+        <v xml:space="preserve">Zone Resilent </v>
       </c>
       <c r="AF15" t="str">
-        <v>Automated by Cloud/SaaS Provider</v>
+        <v>Automated By App</v>
       </c>
       <c r="AG15" t="str">
         <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AH15" t="str">
-        <v>N/A</v>
+        <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AI15" t="str">
-        <v>SaaS Provider</v>
+        <v>HW/SW vendor</v>
       </c>
       <c r="AJ15" t="str">
-        <v>API Monitoring</v>
+        <v>Capacity, Health</v>
       </c>
       <c r="AK15" t="str">
-        <v>Subscription</v>
+        <v>Public Cloud Consumption</v>
       </c>
       <c r="AL15" t="str">
-        <v>OpenAI Pay-as-you-go</v>
+        <v>Seeweb Storage</v>
       </c>
     </row>
     <row r="16">
@@ -7195,85 +7195,85 @@
         <v>PROD</v>
       </c>
       <c r="B16" t="str">
-        <v>99,9%</v>
+        <v>99,5%</v>
       </c>
       <c r="C16" t="str">
-        <v>HA</v>
+        <v>HA-</v>
       </c>
       <c r="D16" t="str">
         <v>AI SERVICES</v>
       </c>
       <c r="E16" t="str">
-        <v>Not W3 Private datacenter</v>
+        <v>Not W3 Public cloud Tenant</v>
       </c>
       <c r="F16" t="str">
         <v>Vendor Private</v>
       </c>
       <c r="G16" t="str">
-        <v>Full IaaS</v>
+        <v>Multi-tenant SaaS</v>
       </c>
       <c r="H16" t="str">
-        <v>W3Suite (Easy Digital Group)</v>
+        <v>OpenAI</v>
       </c>
       <c r="I16" t="str">
-        <v>App (RunTime) - Linux native</v>
+        <v>SaaS  App - Generic Platform</v>
       </c>
       <c r="J16" t="str">
-        <v>2 VPS dedicate</v>
+        <v>SaaS</v>
       </c>
       <c r="K16" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>OpenAI Cloud (EU)</v>
       </c>
       <c r="L16" t="str">
-        <v>Resources - SW configuration</v>
+        <v xml:space="preserve">Internal SaaS/Cloud provider -configuration  </v>
       </c>
       <c r="M16" t="str">
         <v>Active</v>
       </c>
       <c r="N16" t="str">
-        <v>Ops Manual</v>
+        <v>Full Automated</v>
       </c>
       <c r="O16" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+        <v>Native autoscale (SaaS /Cloud providers)</v>
       </c>
       <c r="P16" t="str">
         <v>No outages</v>
       </c>
       <c r="Q16" t="str">
-        <v>Ops - Automated</v>
+        <v>Fully Automated</v>
       </c>
       <c r="R16" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
+        <v>Automated By SaaS/Cloud Provider</v>
       </c>
       <c r="S16" t="str">
         <v>No outages</v>
       </c>
       <c r="T16" t="str">
-        <v>File (Ansible playbook) - VM configuration</v>
+        <v>Database (metadata) - section of application data App configuration</v>
       </c>
       <c r="U16" t="str">
-        <v>SemVer</v>
+        <v>API v1</v>
       </c>
       <c r="V16" t="str">
-        <v>SW Bins</v>
+        <v>N/A</v>
       </c>
       <c r="W16" t="str">
-        <v>Object Store (SW bins)</v>
+        <v>N/A</v>
       </c>
       <c r="X16" t="str">
-        <v>Resource Recovery</v>
+        <v>N/A</v>
       </c>
       <c r="Y16" t="str">
-        <v>On-Premise SW/Appliance</v>
+        <v>N/A</v>
       </c>
       <c r="Z16" t="str">
-        <v>On-premise Store (Appliance)</v>
+        <v>N/A</v>
       </c>
       <c r="AA16" t="str">
-        <v>Daily</v>
+        <v>N/A</v>
       </c>
       <c r="AB16" t="str">
-        <v>1 month</v>
+        <v>N/A</v>
       </c>
       <c r="AC16" t="str">
         <v>N/A</v>
@@ -7282,28 +7282,28 @@
         <v>N/A</v>
       </c>
       <c r="AE16" t="str">
-        <v xml:space="preserve">Local Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF16" t="str">
-        <v>Automated By App</v>
+        <v>Automated by Cloud/SaaS Provider</v>
       </c>
       <c r="AG16" t="str">
         <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AH16" t="str">
-        <v xml:space="preserve">Seconds </v>
+        <v>N/A</v>
       </c>
       <c r="AI16" t="str">
-        <v>SW Integrator</v>
+        <v>SaaS Provider</v>
       </c>
       <c r="AJ16" t="str">
-        <v>AI Routing</v>
+        <v>API Monitoring</v>
       </c>
       <c r="AK16" t="str">
-        <v>Public Cloud Consumption</v>
+        <v>Subscription</v>
       </c>
       <c r="AL16" t="str">
-        <v>Seeweb VPS + W3Suite</v>
+        <v>OpenAI Pay-as-you-go</v>
       </c>
     </row>
     <row r="17">
@@ -7317,7 +7317,7 @@
         <v>HA</v>
       </c>
       <c r="D17" t="str">
-        <v>SECURITY</v>
+        <v>AI SERVICES</v>
       </c>
       <c r="E17" t="str">
         <v>Not W3 Private datacenter</v>
@@ -7335,10 +7335,10 @@
         <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J17" t="str">
-        <v>3 VPS dedicate</v>
+        <v>2 VPC</v>
       </c>
       <c r="K17" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>Seeweb Multinodo Italy (DC1)</v>
       </c>
       <c r="L17" t="str">
         <v>Resources - SW configuration</v>
@@ -7365,7 +7365,7 @@
         <v>No outages</v>
       </c>
       <c r="T17" t="str">
-        <v>Database (metadata) - section of application data App configuration</v>
+        <v>File (Ansible playbook) - VM configuration</v>
       </c>
       <c r="U17" t="str">
         <v>SemVer</v>
@@ -7377,7 +7377,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X17" t="str">
-        <v>Resource: Release and Recovery</v>
+        <v>Resource Recovery</v>
       </c>
       <c r="Y17" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -7392,19 +7392,19 @@
         <v>1 month</v>
       </c>
       <c r="AC17" t="str">
-        <v>1 min</v>
+        <v>N/A</v>
       </c>
       <c r="AD17" t="str">
-        <v>1 week</v>
+        <v>N/A</v>
       </c>
       <c r="AE17" t="str">
-        <v xml:space="preserve">Zone Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF17" t="str">
         <v>Automated By App</v>
       </c>
       <c r="AG17" t="str">
-        <v>Minutes (1-5)</v>
+        <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AH17" t="str">
         <v xml:space="preserve">Seconds </v>
@@ -7413,13 +7413,13 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ17" t="str">
-        <v>Key Rotation, Audit</v>
+        <v>AI Routing</v>
       </c>
       <c r="AK17" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL17" t="str">
-        <v>Seeweb VPS + W3Suite</v>
+        <v>Seeweb VPC + W3Suite</v>
       </c>
     </row>
     <row r="18">
@@ -7427,13 +7427,13 @@
         <v>PROD</v>
       </c>
       <c r="B18" t="str">
-        <v>99,5%</v>
+        <v>99,9%</v>
       </c>
       <c r="C18" t="str">
-        <v>HA-</v>
+        <v>HA</v>
       </c>
       <c r="D18" t="str">
-        <v>OBSERVABILITY</v>
+        <v>SECURITY</v>
       </c>
       <c r="E18" t="str">
         <v>Not W3 Private datacenter</v>
@@ -7445,16 +7445,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H18" t="str">
-        <v>Grafana Labs</v>
+        <v>W3Suite (Easy Digital Group)</v>
       </c>
       <c r="I18" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J18" t="str">
-        <v>2 VPS dedicate</v>
+        <v>3 VPC</v>
       </c>
       <c r="K18" t="str">
-        <v>Seeweb Multinodo Italy</v>
+        <v>Seeweb Multinodo Italy (DC1)</v>
       </c>
       <c r="L18" t="str">
         <v>Resources - SW configuration</v>
@@ -7472,7 +7472,7 @@
         <v>No outages</v>
       </c>
       <c r="Q18" t="str">
-        <v>Ops - Manual</v>
+        <v>Ops - Automated</v>
       </c>
       <c r="R18" t="str">
         <v>Ops Manual - direct Log-on resource</v>
@@ -7481,10 +7481,10 @@
         <v>No outages</v>
       </c>
       <c r="T18" t="str">
-        <v>File (TXT)</v>
+        <v>Database (metadata) - section of application data App configuration</v>
       </c>
       <c r="U18" t="str">
-        <v>10.x</v>
+        <v>SemVer</v>
       </c>
       <c r="V18" t="str">
         <v>SW Bins</v>
@@ -7493,7 +7493,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X18" t="str">
-        <v>Resource Recovery</v>
+        <v>Resource: Release and Recovery</v>
       </c>
       <c r="Y18" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -7508,39 +7508,155 @@
         <v>1 month</v>
       </c>
       <c r="AC18" t="str">
-        <v>N/A</v>
+        <v>1 min</v>
       </c>
       <c r="AD18" t="str">
-        <v>N/A</v>
+        <v>1 week</v>
       </c>
       <c r="AE18" t="str">
-        <v xml:space="preserve">Local Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF18" t="str">
-        <v>Manual By Operation</v>
+        <v>Automated By App</v>
       </c>
       <c r="AG18" t="str">
-        <v>Hour (1-5)</v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AH18" t="str">
-        <v>Hour (1-5)</v>
+        <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AI18" t="str">
         <v>SW Integrator</v>
       </c>
       <c r="AJ18" t="str">
-        <v>Dashboards, Alerts</v>
+        <v>Key Rotation, Audit</v>
       </c>
       <c r="AK18" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL18" t="str">
-        <v>Seeweb VPS</v>
+        <v>Seeweb VPC + W3Suite</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B19" t="str">
+        <v>99,5%</v>
+      </c>
+      <c r="C19" t="str">
+        <v>HA-</v>
+      </c>
+      <c r="D19" t="str">
+        <v>OBSERVABILITY</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Full IaaS</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Grafana Labs</v>
+      </c>
+      <c r="I19" t="str">
+        <v>App (RunTime) - Linux native</v>
+      </c>
+      <c r="J19" t="str">
+        <v>2 VPC</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Seeweb Multinodo Italy (DC1)</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Resources - SW configuration</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Active</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Ops Manual</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+      </c>
+      <c r="P19" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>Ops - Manual</v>
+      </c>
+      <c r="R19" t="str">
+        <v>Ops Manual - direct Log-on resource</v>
+      </c>
+      <c r="S19" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="T19" t="str">
+        <v>File (TXT)</v>
+      </c>
+      <c r="U19" t="str">
+        <v>10.x</v>
+      </c>
+      <c r="V19" t="str">
+        <v>SW Bins</v>
+      </c>
+      <c r="W19" t="str">
+        <v>Object Store (SW bins)</v>
+      </c>
+      <c r="X19" t="str">
+        <v>Resource Recovery</v>
+      </c>
+      <c r="Y19" t="str">
+        <v>On-Premise SW/Appliance</v>
+      </c>
+      <c r="Z19" t="str">
+        <v>On-premise Store (Appliance)</v>
+      </c>
+      <c r="AA19" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="AB19" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC19" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AD19" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AE19" t="str">
+        <v xml:space="preserve">Region Resilent </v>
+      </c>
+      <c r="AF19" t="str">
+        <v>Manual By Operation</v>
+      </c>
+      <c r="AG19" t="str">
+        <v>Hour (1-5)</v>
+      </c>
+      <c r="AH19" t="str">
+        <v>Hour (1-5)</v>
+      </c>
+      <c r="AI19" t="str">
+        <v>SW Integrator</v>
+      </c>
+      <c r="AJ19" t="str">
+        <v>Dashboards, Alerts</v>
+      </c>
+      <c r="AK19" t="str">
+        <v>Public Cloud Consumption</v>
+      </c>
+      <c r="AL19" t="str">
+        <v>Seeweb VPC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A4:AL18"/>
+    <ignoredError numberStoredAsText="1" sqref="A4:AL19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update infrastructure model to accurately reflect cluster setup
Modify the SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx file to align with the actual infrastructure configuration, detailing 7 distinct resources within the Seeweb cluster.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4f3f15ab-59f4-48ee-be3f-90d81d48105b
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
+++ b/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
@@ -5896,6 +5896,12 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C102:C103"/>
+    <mergeCell ref="B256:D256"/>
+    <mergeCell ref="B391:D391"/>
+    <mergeCell ref="B378:D378"/>
+    <mergeCell ref="B368:D368"/>
+    <mergeCell ref="B346:D346"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="B208:D208"/>
@@ -5908,12 +5914,6 @@
     <mergeCell ref="B98:B101"/>
     <mergeCell ref="C98:C101"/>
     <mergeCell ref="B102:B103"/>
-    <mergeCell ref="C102:C103"/>
-    <mergeCell ref="B256:D256"/>
-    <mergeCell ref="B391:D391"/>
-    <mergeCell ref="B378:D378"/>
-    <mergeCell ref="B368:D368"/>
-    <mergeCell ref="B346:D346"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -5924,46 +5924,46 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A4:AL19"/>
+  <dimension ref="A4:AL14"/>
   <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="26.83203125" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" customWidth="1"/>
-    <col min="6" max="6" width="26.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
-    <col min="9" max="9" width="26.83203125" customWidth="1"/>
-    <col min="10" max="10" width="26.83203125" customWidth="1"/>
-    <col min="11" max="11" width="26.83203125" customWidth="1"/>
-    <col min="12" max="12" width="26.83203125" customWidth="1"/>
-    <col min="13" max="13" width="26.83203125" customWidth="1"/>
-    <col min="14" max="14" width="26.83203125" customWidth="1"/>
-    <col min="15" max="15" width="26.83203125" customWidth="1"/>
-    <col min="16" max="16" width="26.83203125" customWidth="1"/>
-    <col min="17" max="17" width="26.83203125" customWidth="1"/>
-    <col min="18" max="18" width="26.83203125" customWidth="1"/>
-    <col min="19" max="19" width="26.83203125" customWidth="1"/>
-    <col min="20" max="20" width="26.83203125" customWidth="1"/>
-    <col min="21" max="21" width="26.83203125" customWidth="1"/>
-    <col min="22" max="22" width="26.83203125" customWidth="1"/>
-    <col min="23" max="23" width="26.83203125" customWidth="1"/>
-    <col min="24" max="24" width="26.83203125" customWidth="1"/>
-    <col min="25" max="25" width="26.83203125" customWidth="1"/>
-    <col min="26" max="26" width="26.83203125" customWidth="1"/>
-    <col min="27" max="27" width="26.83203125" customWidth="1"/>
-    <col min="28" max="28" width="26.83203125" customWidth="1"/>
-    <col min="29" max="29" width="26.83203125" customWidth="1"/>
-    <col min="30" max="30" width="26.83203125" customWidth="1"/>
-    <col min="31" max="31" width="26.83203125" customWidth="1"/>
-    <col min="32" max="32" width="26.83203125" customWidth="1"/>
-    <col min="33" max="33" width="26.83203125" customWidth="1"/>
-    <col min="34" max="34" width="26.83203125" customWidth="1"/>
-    <col min="35" max="35" width="26.83203125" customWidth="1"/>
-    <col min="36" max="36" width="26.83203125" customWidth="1"/>
-    <col min="37" max="37" width="26.83203125" customWidth="1"/>
-    <col min="38" max="38" width="26.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="28.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="28.83203125" customWidth="1"/>
+    <col min="10" max="10" width="28.83203125" customWidth="1"/>
+    <col min="11" max="11" width="28.83203125" customWidth="1"/>
+    <col min="12" max="12" width="28.83203125" customWidth="1"/>
+    <col min="13" max="13" width="28.83203125" customWidth="1"/>
+    <col min="14" max="14" width="28.83203125" customWidth="1"/>
+    <col min="15" max="15" width="28.83203125" customWidth="1"/>
+    <col min="16" max="16" width="28.83203125" customWidth="1"/>
+    <col min="17" max="17" width="28.83203125" customWidth="1"/>
+    <col min="18" max="18" width="28.83203125" customWidth="1"/>
+    <col min="19" max="19" width="28.83203125" customWidth="1"/>
+    <col min="20" max="20" width="28.83203125" customWidth="1"/>
+    <col min="21" max="21" width="28.83203125" customWidth="1"/>
+    <col min="22" max="22" width="28.83203125" customWidth="1"/>
+    <col min="23" max="23" width="28.83203125" customWidth="1"/>
+    <col min="24" max="24" width="28.83203125" customWidth="1"/>
+    <col min="25" max="25" width="28.83203125" customWidth="1"/>
+    <col min="26" max="26" width="28.83203125" customWidth="1"/>
+    <col min="27" max="27" width="28.83203125" customWidth="1"/>
+    <col min="28" max="28" width="28.83203125" customWidth="1"/>
+    <col min="29" max="29" width="28.83203125" customWidth="1"/>
+    <col min="30" max="30" width="28.83203125" customWidth="1"/>
+    <col min="31" max="31" width="28.83203125" customWidth="1"/>
+    <col min="32" max="32" width="28.83203125" customWidth="1"/>
+    <col min="33" max="33" width="28.83203125" customWidth="1"/>
+    <col min="34" max="34" width="28.83203125" customWidth="1"/>
+    <col min="35" max="35" width="28.83203125" customWidth="1"/>
+    <col min="36" max="36" width="28.83203125" customWidth="1"/>
+    <col min="37" max="37" width="28.83203125" customWidth="1"/>
+    <col min="38" max="38" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4">
@@ -6273,7 +6273,7 @@
         <v>HA</v>
       </c>
       <c r="D8" t="str">
-        <v>CORE PLATFORM</v>
+        <v>INFRASTRUCTURE</v>
       </c>
       <c r="E8" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6285,16 +6285,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H8" t="str">
-        <v>Seeweb S.r.l. + Proxmox VE</v>
+        <v>Seeweb S.r.l.</v>
       </c>
       <c r="I8" t="str">
         <v>Virtualization Platform - ProxMox</v>
       </c>
       <c r="J8" t="str">
-        <v>Multinodo Cluster</v>
+        <v>1 Cluster Multinodo</v>
       </c>
       <c r="K8" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
+        <v>Seeweb Italy (DC1)</v>
       </c>
       <c r="L8" t="str">
         <v>Resources - SW configuration</v>
@@ -6324,7 +6324,7 @@
         <v>File (TXT)</v>
       </c>
       <c r="U8" t="str">
-        <v>8.1.x</v>
+        <v>Proxmox VE 8.x</v>
       </c>
       <c r="V8" t="str">
         <v>VMI (virtual Machine Image) - KVM</v>
@@ -6369,13 +6369,13 @@
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ8" t="str">
-        <v>VM Mgmt, PBS Replication</v>
+        <v>Cluster Management</v>
       </c>
       <c r="AK8" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL8" t="str">
-        <v>Seeweb Multinodo + PBS</v>
+        <v>Seeweb Multinodo Contract</v>
       </c>
     </row>
     <row r="9">
@@ -6383,13 +6383,13 @@
         <v>PROD</v>
       </c>
       <c r="B9" t="str">
-        <v>99,9%</v>
+        <v>99,5%</v>
       </c>
       <c r="C9" t="str">
-        <v>HA</v>
+        <v>HA-</v>
       </c>
       <c r="D9" t="str">
-        <v>CORE PLATFORM</v>
+        <v>INFRASTRUCTURE</v>
       </c>
       <c r="E9" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6398,19 +6398,19 @@
         <v>Vendor Private</v>
       </c>
       <c r="G9" t="str">
-        <v>Full IaaS</v>
+        <v>HW Appliance</v>
       </c>
       <c r="H9" t="str">
-        <v>Proxmox Server Solutions GmbH</v>
+        <v>Seeweb S.r.l. (Fortinet)</v>
       </c>
       <c r="I9" t="str">
-        <v>Bare Metal-Linux OS</v>
+        <v>HW Appliance - FortiGate NGFW</v>
       </c>
       <c r="J9" t="str">
-        <v>1 (Dedicato)</v>
+        <v>1 (Single)</v>
       </c>
       <c r="K9" t="str">
-        <v>Seeweb Italy (DC2 - DR Site)</v>
+        <v>Seeweb Italy (DC1)</v>
       </c>
       <c r="L9" t="str">
         <v>Resources - SW configuration</v>
@@ -6419,10 +6419,10 @@
         <v>Active</v>
       </c>
       <c r="N9" t="str">
-        <v>Ops Manual</v>
+        <v>Fixed capacity</v>
       </c>
       <c r="O9" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+        <v>Do not scale - Fixed capacity</v>
       </c>
       <c r="P9" t="str">
         <v>No outages</v>
@@ -6440,13 +6440,13 @@
         <v>File (TXT)</v>
       </c>
       <c r="U9" t="str">
-        <v>3.x</v>
+        <v>FortiOS 7.x</v>
       </c>
       <c r="V9" t="str">
         <v>SW Bins</v>
       </c>
       <c r="W9" t="str">
-        <v>Object Store (SW bins)</v>
+        <v>Private Others Registry</v>
       </c>
       <c r="X9" t="str">
         <v>Resource Recovery</v>
@@ -6464,13 +6464,13 @@
         <v>1 month</v>
       </c>
       <c r="AC9" t="str">
-        <v>1 min</v>
+        <v>N/A</v>
       </c>
       <c r="AD9" t="str">
-        <v>1 week</v>
+        <v>N/A</v>
       </c>
       <c r="AE9" t="str">
-        <v xml:space="preserve">Region Resilent </v>
+        <v xml:space="preserve">Local Resilent </v>
       </c>
       <c r="AF9" t="str">
         <v>Manual By Operation</v>
@@ -6479,19 +6479,19 @@
         <v>Hour (1-5)</v>
       </c>
       <c r="AH9" t="str">
-        <v>Minutes (1-5)</v>
+        <v>Hour (1-5)</v>
       </c>
       <c r="AI9" t="str">
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ9" t="str">
-        <v>Backup Storage, DR</v>
+        <v>Security Management</v>
       </c>
       <c r="AK9" t="str">
-        <v>Public Cloud Consumption</v>
+        <v>COTs SW License</v>
       </c>
       <c r="AL9" t="str">
-        <v>Seeweb PBS Dedicated</v>
+        <v>Seeweb FortiGate Service</v>
       </c>
     </row>
     <row r="10">
@@ -6499,13 +6499,13 @@
         <v>PROD</v>
       </c>
       <c r="B10" t="str">
-        <v>99,5%</v>
+        <v>99,9%</v>
       </c>
       <c r="C10" t="str">
-        <v>HA-</v>
+        <v>HA</v>
       </c>
       <c r="D10" t="str">
-        <v>CORE PLATFORM</v>
+        <v>INFRASTRUCTURE</v>
       </c>
       <c r="E10" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6514,19 +6514,19 @@
         <v>Vendor Private</v>
       </c>
       <c r="G10" t="str">
-        <v>HW Appliance</v>
+        <v>Bare Metal</v>
       </c>
       <c r="H10" t="str">
-        <v>Fortinet Inc.</v>
+        <v>Seeweb S.r.l.</v>
       </c>
       <c r="I10" t="str">
-        <v>HW Appliance - FortiGate NGFW</v>
+        <v>Bare Metal-Linux OS</v>
       </c>
       <c r="J10" t="str">
-        <v>1 (Single)</v>
+        <v>1 (Dedicato)</v>
       </c>
       <c r="K10" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
+        <v>Seeweb Italy (DC2 - DR)</v>
       </c>
       <c r="L10" t="str">
         <v>Resources - SW configuration</v>
@@ -6535,10 +6535,10 @@
         <v>Active</v>
       </c>
       <c r="N10" t="str">
-        <v>Fixed capacity</v>
+        <v>Ops Manual</v>
       </c>
       <c r="O10" t="str">
-        <v>Do not scale - Fixed capacity</v>
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P10" t="str">
         <v>No outages</v>
@@ -6556,13 +6556,13 @@
         <v>File (TXT)</v>
       </c>
       <c r="U10" t="str">
-        <v>7.4.x</v>
+        <v>PBS 3.x</v>
       </c>
       <c r="V10" t="str">
         <v>SW Bins</v>
       </c>
       <c r="W10" t="str">
-        <v>Private Others Registry</v>
+        <v>Object Store (SW bins)</v>
       </c>
       <c r="X10" t="str">
         <v>Resource Recovery</v>
@@ -6580,13 +6580,13 @@
         <v>1 month</v>
       </c>
       <c r="AC10" t="str">
-        <v>N/A</v>
+        <v>1 min</v>
       </c>
       <c r="AD10" t="str">
-        <v>N/A</v>
+        <v>1 week</v>
       </c>
       <c r="AE10" t="str">
-        <v xml:space="preserve">Local Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF10" t="str">
         <v>Manual By Operation</v>
@@ -6595,19 +6595,19 @@
         <v>Hour (1-5)</v>
       </c>
       <c r="AH10" t="str">
-        <v>Hour (1-5)</v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AI10" t="str">
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ10" t="str">
-        <v>Security, Monitoring</v>
+        <v>Backup &amp; DR</v>
       </c>
       <c r="AK10" t="str">
-        <v>COTs SW License</v>
+        <v>Public Cloud Consumption</v>
       </c>
       <c r="AL10" t="str">
-        <v>FortiCare + FortiGuard</v>
+        <v>Seeweb PBS Service</v>
       </c>
     </row>
     <row r="11">
@@ -6621,7 +6621,7 @@
         <v>HA</v>
       </c>
       <c r="D11" t="str">
-        <v>CORE PLATFORM</v>
+        <v>APPLICATION</v>
       </c>
       <c r="E11" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6633,16 +6633,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H11" t="str">
-        <v>W3Suite (Easy Digital Group)</v>
+        <v>Seeweb S.r.l.</v>
       </c>
       <c r="I11" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J11" t="str">
-        <v>3 VPC</v>
+        <v>1 VPC (Nginx + LB)</v>
       </c>
       <c r="K11" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
+        <v>Seeweb Italy (DC1)</v>
       </c>
       <c r="L11" t="str">
         <v>Resources - SW configuration</v>
@@ -6672,7 +6672,7 @@
         <v>File (Ansible playbook) - VM configuration</v>
       </c>
       <c r="U11" t="str">
-        <v>SemVer</v>
+        <v>Nginx 1.24 + W3Suite FE</v>
       </c>
       <c r="V11" t="str">
         <v>SW Bins</v>
@@ -6708,22 +6708,22 @@
         <v>Automated By App</v>
       </c>
       <c r="AG11" t="str">
-        <v>Minutes (1-5)</v>
+        <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AH11" t="str">
-        <v xml:space="preserve">Seconds </v>
+        <v>N/A</v>
       </c>
       <c r="AI11" t="str">
         <v>SW Integrator</v>
       </c>
       <c r="AJ11" t="str">
-        <v>Deploy, Monitoring</v>
+        <v>TLS, Routing, LB Config</v>
       </c>
       <c r="AK11" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL11" t="str">
-        <v>Seeweb VPC + W3Suite</v>
+        <v>Seeweb VPC</v>
       </c>
     </row>
     <row r="12">
@@ -6737,7 +6737,7 @@
         <v>HA</v>
       </c>
       <c r="D12" t="str">
-        <v>CORE PLATFORM</v>
+        <v>APPLICATION</v>
       </c>
       <c r="E12" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6749,16 +6749,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H12" t="str">
-        <v>F5 Networks (Nginx)</v>
+        <v>Seeweb S.r.l.</v>
       </c>
       <c r="I12" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J12" t="str">
-        <v>2 VPC</v>
+        <v>1 VPC (API+Redis+MCP)</v>
       </c>
       <c r="K12" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
+        <v>Seeweb Italy (DC1)</v>
       </c>
       <c r="L12" t="str">
         <v>Resources - SW configuration</v>
@@ -6776,7 +6776,7 @@
         <v>No outages</v>
       </c>
       <c r="Q12" t="str">
-        <v>Ops - Manual</v>
+        <v>Ops - Automated</v>
       </c>
       <c r="R12" t="str">
         <v>Ops Manual - direct Log-on resource</v>
@@ -6785,10 +6785,10 @@
         <v>No outages</v>
       </c>
       <c r="T12" t="str">
-        <v>File (TXT)</v>
+        <v>File (Ansible playbook) - VM configuration</v>
       </c>
       <c r="U12" t="str">
-        <v>1.24.x</v>
+        <v>W3Suite API + Redis + MCP</v>
       </c>
       <c r="V12" t="str">
         <v>SW Bins</v>
@@ -6812,10 +6812,10 @@
         <v>1 month</v>
       </c>
       <c r="AC12" t="str">
-        <v>N/A</v>
+        <v>1 min</v>
       </c>
       <c r="AD12" t="str">
-        <v>N/A</v>
+        <v>1 week</v>
       </c>
       <c r="AE12" t="str">
         <v xml:space="preserve">Region Resilent </v>
@@ -6824,16 +6824,16 @@
         <v>Automated By App</v>
       </c>
       <c r="AG12" t="str">
+        <v>Minutes (1-5)</v>
+      </c>
+      <c r="AH12" t="str">
         <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AH12" t="str">
-        <v>N/A</v>
       </c>
       <c r="AI12" t="str">
         <v>SW Integrator</v>
       </c>
       <c r="AJ12" t="str">
-        <v>TLS, Config</v>
+        <v>Deploy, API, AI Gateway</v>
       </c>
       <c r="AK12" t="str">
         <v>Public Cloud Consumption</v>
@@ -6853,7 +6853,7 @@
         <v>HA</v>
       </c>
       <c r="D13" t="str">
-        <v>CORE PLATFORM</v>
+        <v>DATABASE</v>
       </c>
       <c r="E13" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6865,16 +6865,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H13" t="str">
-        <v>Redis Ltd</v>
+        <v>Seeweb S.r.l.</v>
       </c>
       <c r="I13" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J13" t="str">
-        <v>2 VPC</v>
+        <v>1 VPC (PostgreSQL Primary)</v>
       </c>
       <c r="K13" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
+        <v>Seeweb Italy (DC1)</v>
       </c>
       <c r="L13" t="str">
         <v>Resources - SW configuration</v>
@@ -6889,7 +6889,7 @@
         <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P13" t="str">
-        <v>No outages</v>
+        <v>Minutes (1-10)</v>
       </c>
       <c r="Q13" t="str">
         <v>Ops - Manual</v>
@@ -6898,13 +6898,13 @@
         <v>Ops Manual - direct Log-on resource</v>
       </c>
       <c r="S13" t="str">
-        <v>No outages</v>
+        <v>Minutes (1-10)</v>
       </c>
       <c r="T13" t="str">
         <v>File (TXT)</v>
       </c>
       <c r="U13" t="str">
-        <v>7.2.x</v>
+        <v>PostgreSQL 15.x</v>
       </c>
       <c r="V13" t="str">
         <v>SW Bins</v>
@@ -6913,7 +6913,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X13" t="str">
-        <v>Resource Recovery</v>
+        <v>Resource: Release and Recovery</v>
       </c>
       <c r="Y13" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -6940,7 +6940,7 @@
         <v>Automated By App</v>
       </c>
       <c r="AG13" t="str">
-        <v xml:space="preserve">Seconds </v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AH13" t="str">
         <v xml:space="preserve">Seconds </v>
@@ -6949,7 +6949,7 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ13" t="str">
-        <v>Memory Monitoring</v>
+        <v>Backup, Tuning, PITR</v>
       </c>
       <c r="AK13" t="str">
         <v>Public Cloud Consumption</v>
@@ -6969,7 +6969,7 @@
         <v>HA</v>
       </c>
       <c r="D14" t="str">
-        <v>DATABASE LAYER</v>
+        <v>DATABASE</v>
       </c>
       <c r="E14" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6981,22 +6981,22 @@
         <v>Full IaaS</v>
       </c>
       <c r="H14" t="str">
-        <v>PostgreSQL Global Development Group</v>
+        <v>Seeweb S.r.l.</v>
       </c>
       <c r="I14" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
       <c r="J14" t="str">
-        <v>2 VPC (Primary+Replica)</v>
+        <v>1 VPC (PostgreSQL Replica)</v>
       </c>
       <c r="K14" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
+        <v>Seeweb Italy (DC1)</v>
       </c>
       <c r="L14" t="str">
         <v>Resources - SW configuration</v>
       </c>
       <c r="M14" t="str">
-        <v>Active</v>
+        <v>Standby</v>
       </c>
       <c r="N14" t="str">
         <v>Ops Manual</v>
@@ -7005,7 +7005,7 @@
         <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P14" t="str">
-        <v>Minutes (1-10)</v>
+        <v>No outages</v>
       </c>
       <c r="Q14" t="str">
         <v>Ops - Manual</v>
@@ -7014,13 +7014,13 @@
         <v>Ops Manual - direct Log-on resource</v>
       </c>
       <c r="S14" t="str">
-        <v>Minutes (1-10)</v>
+        <v>No outages</v>
       </c>
       <c r="T14" t="str">
         <v>File (TXT)</v>
       </c>
       <c r="U14" t="str">
-        <v>15.x</v>
+        <v>PostgreSQL 15.x</v>
       </c>
       <c r="V14" t="str">
         <v>SW Bins</v>
@@ -7029,7 +7029,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X14" t="str">
-        <v>Resource: Release and Recovery</v>
+        <v>Resource Recovery</v>
       </c>
       <c r="Y14" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -7056,7 +7056,7 @@
         <v>Automated By App</v>
       </c>
       <c r="AG14" t="str">
-        <v>Minutes (1-5)</v>
+        <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AH14" t="str">
         <v xml:space="preserve">Seconds </v>
@@ -7065,7 +7065,7 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ14" t="str">
-        <v>Backup, Tuning, PITR</v>
+        <v>Streaming Replication</v>
       </c>
       <c r="AK14" t="str">
         <v>Public Cloud Consumption</v>
@@ -7074,589 +7074,9 @@
         <v>Seeweb VPC</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B15" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C15" t="str">
-        <v>HA</v>
-      </c>
-      <c r="D15" t="str">
-        <v>DATABASE LAYER</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G15" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H15" t="str">
-        <v>Seeweb S.r.l. (Ceph Storage)</v>
-      </c>
-      <c r="I15" t="str">
-        <v>Bare Metal-Linux OS</v>
-      </c>
-      <c r="J15" t="str">
-        <v>Cluster Ceph</v>
-      </c>
-      <c r="K15" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
-      </c>
-      <c r="L15" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M15" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N15" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O15" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P15" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q15" t="str">
-        <v>Ops - Manual</v>
-      </c>
-      <c r="R15" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S15" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T15" t="str">
-        <v>File (TXT)</v>
-      </c>
-      <c r="U15" t="str">
-        <v>Quincy</v>
-      </c>
-      <c r="V15" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W15" t="str">
-        <v>Object Store (SW bins)</v>
-      </c>
-      <c r="X15" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y15" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z15" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA15" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB15" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC15" t="str">
-        <v>1 min</v>
-      </c>
-      <c r="AD15" t="str">
-        <v>1 week</v>
-      </c>
-      <c r="AE15" t="str">
-        <v xml:space="preserve">Zone Resilent </v>
-      </c>
-      <c r="AF15" t="str">
-        <v>Automated By App</v>
-      </c>
-      <c r="AG15" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AH15" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AI15" t="str">
-        <v>HW/SW vendor</v>
-      </c>
-      <c r="AJ15" t="str">
-        <v>Capacity, Health</v>
-      </c>
-      <c r="AK15" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL15" t="str">
-        <v>Seeweb Storage</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B16" t="str">
-        <v>99,5%</v>
-      </c>
-      <c r="C16" t="str">
-        <v>HA-</v>
-      </c>
-      <c r="D16" t="str">
-        <v>AI SERVICES</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Not W3 Public cloud Tenant</v>
-      </c>
-      <c r="F16" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G16" t="str">
-        <v>Multi-tenant SaaS</v>
-      </c>
-      <c r="H16" t="str">
-        <v>OpenAI</v>
-      </c>
-      <c r="I16" t="str">
-        <v>SaaS  App - Generic Platform</v>
-      </c>
-      <c r="J16" t="str">
-        <v>SaaS</v>
-      </c>
-      <c r="K16" t="str">
-        <v>OpenAI Cloud (EU)</v>
-      </c>
-      <c r="L16" t="str">
-        <v xml:space="preserve">Internal SaaS/Cloud provider -configuration  </v>
-      </c>
-      <c r="M16" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N16" t="str">
-        <v>Full Automated</v>
-      </c>
-      <c r="O16" t="str">
-        <v>Native autoscale (SaaS /Cloud providers)</v>
-      </c>
-      <c r="P16" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q16" t="str">
-        <v>Fully Automated</v>
-      </c>
-      <c r="R16" t="str">
-        <v>Automated By SaaS/Cloud Provider</v>
-      </c>
-      <c r="S16" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T16" t="str">
-        <v>Database (metadata) - section of application data App configuration</v>
-      </c>
-      <c r="U16" t="str">
-        <v>API v1</v>
-      </c>
-      <c r="V16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="W16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="X16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="Y16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="Z16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AA16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AB16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AC16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AD16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AE16" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF16" t="str">
-        <v>Automated by Cloud/SaaS Provider</v>
-      </c>
-      <c r="AG16" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AH16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AI16" t="str">
-        <v>SaaS Provider</v>
-      </c>
-      <c r="AJ16" t="str">
-        <v>API Monitoring</v>
-      </c>
-      <c r="AK16" t="str">
-        <v>Subscription</v>
-      </c>
-      <c r="AL16" t="str">
-        <v>OpenAI Pay-as-you-go</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B17" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C17" t="str">
-        <v>HA</v>
-      </c>
-      <c r="D17" t="str">
-        <v>AI SERVICES</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F17" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G17" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H17" t="str">
-        <v>W3Suite (Easy Digital Group)</v>
-      </c>
-      <c r="I17" t="str">
-        <v>App (RunTime) - Linux native</v>
-      </c>
-      <c r="J17" t="str">
-        <v>2 VPC</v>
-      </c>
-      <c r="K17" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
-      </c>
-      <c r="L17" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M17" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N17" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O17" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P17" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q17" t="str">
-        <v>Ops - Automated</v>
-      </c>
-      <c r="R17" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S17" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T17" t="str">
-        <v>File (Ansible playbook) - VM configuration</v>
-      </c>
-      <c r="U17" t="str">
-        <v>SemVer</v>
-      </c>
-      <c r="V17" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W17" t="str">
-        <v>Object Store (SW bins)</v>
-      </c>
-      <c r="X17" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y17" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z17" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA17" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB17" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC17" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AD17" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AE17" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF17" t="str">
-        <v>Automated By App</v>
-      </c>
-      <c r="AG17" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AH17" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AI17" t="str">
-        <v>SW Integrator</v>
-      </c>
-      <c r="AJ17" t="str">
-        <v>AI Routing</v>
-      </c>
-      <c r="AK17" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL17" t="str">
-        <v>Seeweb VPC + W3Suite</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B18" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C18" t="str">
-        <v>HA</v>
-      </c>
-      <c r="D18" t="str">
-        <v>SECURITY</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F18" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G18" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H18" t="str">
-        <v>W3Suite (Easy Digital Group)</v>
-      </c>
-      <c r="I18" t="str">
-        <v>App (RunTime) - Linux native</v>
-      </c>
-      <c r="J18" t="str">
-        <v>3 VPC</v>
-      </c>
-      <c r="K18" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
-      </c>
-      <c r="L18" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M18" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N18" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O18" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P18" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q18" t="str">
-        <v>Ops - Automated</v>
-      </c>
-      <c r="R18" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S18" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T18" t="str">
-        <v>Database (metadata) - section of application data App configuration</v>
-      </c>
-      <c r="U18" t="str">
-        <v>SemVer</v>
-      </c>
-      <c r="V18" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W18" t="str">
-        <v>Object Store (SW bins)</v>
-      </c>
-      <c r="X18" t="str">
-        <v>Resource: Release and Recovery</v>
-      </c>
-      <c r="Y18" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z18" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA18" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB18" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC18" t="str">
-        <v>1 min</v>
-      </c>
-      <c r="AD18" t="str">
-        <v>1 week</v>
-      </c>
-      <c r="AE18" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF18" t="str">
-        <v>Automated By App</v>
-      </c>
-      <c r="AG18" t="str">
-        <v>Minutes (1-5)</v>
-      </c>
-      <c r="AH18" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AI18" t="str">
-        <v>SW Integrator</v>
-      </c>
-      <c r="AJ18" t="str">
-        <v>Key Rotation, Audit</v>
-      </c>
-      <c r="AK18" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL18" t="str">
-        <v>Seeweb VPC + W3Suite</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B19" t="str">
-        <v>99,5%</v>
-      </c>
-      <c r="C19" t="str">
-        <v>HA-</v>
-      </c>
-      <c r="D19" t="str">
-        <v>OBSERVABILITY</v>
-      </c>
-      <c r="E19" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F19" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G19" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H19" t="str">
-        <v>Grafana Labs</v>
-      </c>
-      <c r="I19" t="str">
-        <v>App (RunTime) - Linux native</v>
-      </c>
-      <c r="J19" t="str">
-        <v>2 VPC</v>
-      </c>
-      <c r="K19" t="str">
-        <v>Seeweb Multinodo Italy (DC1)</v>
-      </c>
-      <c r="L19" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M19" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N19" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O19" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P19" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q19" t="str">
-        <v>Ops - Manual</v>
-      </c>
-      <c r="R19" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S19" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T19" t="str">
-        <v>File (TXT)</v>
-      </c>
-      <c r="U19" t="str">
-        <v>10.x</v>
-      </c>
-      <c r="V19" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W19" t="str">
-        <v>Object Store (SW bins)</v>
-      </c>
-      <c r="X19" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y19" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z19" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA19" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB19" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC19" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AD19" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AE19" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF19" t="str">
-        <v>Manual By Operation</v>
-      </c>
-      <c r="AG19" t="str">
-        <v>Hour (1-5)</v>
-      </c>
-      <c r="AH19" t="str">
-        <v>Hour (1-5)</v>
-      </c>
-      <c r="AI19" t="str">
-        <v>SW Integrator</v>
-      </c>
-      <c r="AJ19" t="str">
-        <v>Dashboards, Alerts</v>
-      </c>
-      <c r="AK19" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL19" t="str">
-        <v>Seeweb VPC</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A4:AL19"/>
+    <ignoredError numberStoredAsText="1" sqref="A4:AL14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update service resource model spreadsheet with infrastructure details
Update the SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx file to accurately reflect the infrastructure details, including resource distribution and technical models, as per the final analysis of the W3Suite architecture within the Seeweb environment.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a91904ee-5886-46c0-8237-da77a089e5b0
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
+++ b/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
@@ -7,9 +7,9 @@
     <sheet name="Proposal Structure" sheetId="2" r:id="rId2"/>
     <sheet name="Resource Model" sheetId="3" r:id="rId3"/>
     <sheet name=" Service Model Example" sheetId="4" r:id="rId4"/>
-    <sheet name="Service Resource Distribution" sheetId="5" r:id="rId5"/>
-    <sheet name="Values&amp;Descriptions" sheetId="6" r:id="rId6"/>
-    <sheet name=" Service Model (to be filled)" sheetId="7" r:id="rId7"/>
+    <sheet name="Values&amp;Descriptions" sheetId="5" r:id="rId5"/>
+    <sheet name=" Service Model (to be filled)" sheetId="6" r:id="rId6"/>
+    <sheet name="Service Resource Distribution" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -2496,154 +2496,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="C1:S12"/>
-  <sheetData>
-    <row r="2">
-      <c r="C2" t="str">
-        <v>Public Cloud Zones or W3 Sites</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
-      <c r="C3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Field Definition &amp; Values _x000d_
-_x000d_
-Module of solution</v>
-      </c>
-      <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Field Definition &amp; Values _x000d_
-_x000d_
-Resource of module</v>
-      </c>
-      <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Field Definition &amp; Values_x000d_
-Resource component_x000d_
-Enables to specify (if needed) components of the resources that are assigned to a site, that corrspond to different configuration_x000d_
-The resources intsalled on the site can have differen configuration that is worth to describe_x000d_
-_x000d_
-Example xample 5G Platform has specific configuration (means which cNF are  deployed or not in the istance of specific  site._x000d_
-_x000d_
-For cloud deployment for example a standBy resource can have diffrent configration</v>
-      </c>
-      <c r="F3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Field Definition &amp; Values_x000d_
-_x000d_
-W3 Sites List_x000d_
-</v>
-      </c>
-    </row>
-    <row r="7" xml:space="preserve">
-      <c r="C7" t="str">
-        <v>Module</v>
-      </c>
-      <c r="D7" t="str" xml:space="preserve">
-        <v xml:space="preserve">Service_x000d_
-Resources</v>
-      </c>
-      <c r="E7" t="str" xml:space="preserve">
-        <v xml:space="preserve">Resource _x000d_
-Component (if needed)</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Region (Zone/site)</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="I7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="J7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="M7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="N7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="O7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="P7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="Q7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="R7" t="str">
-        <v>Zone/site</v>
-      </c>
-      <c r="S7" t="str">
-        <v>Zone/site</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="F8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="G8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="H8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="I8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="J8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="K8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="L8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="M8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="N8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="O8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="P8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="Q8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="R8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-      <c r="S8" t="str">
-        <v>W3-(Core site) - 1</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="F3:S3"/>
-    <mergeCell ref="C2:S2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="C1:S12"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:H395"/>
   <sheetData>
     <row r="2">
@@ -5922,460 +5774,354 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A4:AL14"/>
+  <dimension ref="A1:AL15"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="28.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.83203125" customWidth="1"/>
-    <col min="8" max="8" width="28.83203125" customWidth="1"/>
-    <col min="9" max="9" width="28.83203125" customWidth="1"/>
-    <col min="10" max="10" width="28.83203125" customWidth="1"/>
-    <col min="11" max="11" width="28.83203125" customWidth="1"/>
-    <col min="12" max="12" width="28.83203125" customWidth="1"/>
-    <col min="13" max="13" width="28.83203125" customWidth="1"/>
-    <col min="14" max="14" width="28.83203125" customWidth="1"/>
-    <col min="15" max="15" width="28.83203125" customWidth="1"/>
-    <col min="16" max="16" width="28.83203125" customWidth="1"/>
-    <col min="17" max="17" width="28.83203125" customWidth="1"/>
-    <col min="18" max="18" width="28.83203125" customWidth="1"/>
-    <col min="19" max="19" width="28.83203125" customWidth="1"/>
-    <col min="20" max="20" width="28.83203125" customWidth="1"/>
-    <col min="21" max="21" width="28.83203125" customWidth="1"/>
-    <col min="22" max="22" width="28.83203125" customWidth="1"/>
-    <col min="23" max="23" width="28.83203125" customWidth="1"/>
-    <col min="24" max="24" width="28.83203125" customWidth="1"/>
-    <col min="25" max="25" width="28.83203125" customWidth="1"/>
-    <col min="26" max="26" width="28.83203125" customWidth="1"/>
-    <col min="27" max="27" width="28.83203125" customWidth="1"/>
-    <col min="28" max="28" width="28.83203125" customWidth="1"/>
-    <col min="29" max="29" width="28.83203125" customWidth="1"/>
-    <col min="30" max="30" width="28.83203125" customWidth="1"/>
-    <col min="31" max="31" width="28.83203125" customWidth="1"/>
-    <col min="32" max="32" width="28.83203125" customWidth="1"/>
-    <col min="33" max="33" width="28.83203125" customWidth="1"/>
-    <col min="34" max="34" width="28.83203125" customWidth="1"/>
-    <col min="35" max="35" width="28.83203125" customWidth="1"/>
-    <col min="36" max="36" width="28.83203125" customWidth="1"/>
-    <col min="37" max="37" width="28.83203125" customWidth="1"/>
-    <col min="38" max="38" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="22.83203125" customWidth="1"/>
+    <col min="14" max="14" width="22.83203125" customWidth="1"/>
+    <col min="15" max="15" width="22.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
+    <col min="17" max="17" width="22.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" customWidth="1"/>
+    <col min="21" max="21" width="22.83203125" customWidth="1"/>
+    <col min="22" max="22" width="22.83203125" customWidth="1"/>
+    <col min="23" max="23" width="22.83203125" customWidth="1"/>
+    <col min="24" max="24" width="22.83203125" customWidth="1"/>
+    <col min="25" max="25" width="22.83203125" customWidth="1"/>
+    <col min="26" max="26" width="22.83203125" customWidth="1"/>
+    <col min="27" max="27" width="22.83203125" customWidth="1"/>
+    <col min="28" max="28" width="22.83203125" customWidth="1"/>
+    <col min="29" max="29" width="22.83203125" customWidth="1"/>
+    <col min="30" max="30" width="22.83203125" customWidth="1"/>
+    <col min="31" max="31" width="22.83203125" customWidth="1"/>
+    <col min="32" max="32" width="22.83203125" customWidth="1"/>
+    <col min="33" max="33" width="22.83203125" customWidth="1"/>
+    <col min="34" max="34" width="22.83203125" customWidth="1"/>
+    <col min="35" max="35" width="22.83203125" customWidth="1"/>
+    <col min="36" max="36" width="22.83203125" customWidth="1"/>
+    <col min="37" max="37" width="22.83203125" customWidth="1"/>
+    <col min="38" max="38" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>HERE YOU CAN FIND SOME NOTES TO HELP YOU UNDERSTAND HOW TO FILL IN THIS FORM. YOU CAN FIND THE COMPLETE VALUES LIST AND RELATED DESCRIPTION ON TAB "Values&amp;Description"</v>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="str">
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Environment</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SLA Model &amp; Resource Model</v>
+      </c>
+      <c r="C5" t="str">
         <v/>
       </c>
-      <c r="B4" t="str">
-        <v>Environment</v>
-      </c>
-      <c r="C4" t="str">
-        <v>SLA Model &amp; Resource Model</v>
-      </c>
-      <c r="D4" t="str">
+      <c r="D5" t="str">
         <v/>
       </c>
-      <c r="E4" t="str">
+      <c r="E5" t="str">
         <v/>
       </c>
-      <c r="F4" t="str">
+      <c r="F5" t="str">
         <v/>
       </c>
-      <c r="G4" t="str">
+      <c r="G5" t="str">
         <v/>
       </c>
-      <c r="H4" t="str">
+      <c r="H5" t="str">
         <v/>
       </c>
-      <c r="I4" t="str">
+      <c r="I5" t="str">
         <v/>
       </c>
-      <c r="J4" t="str">
+      <c r="J5" t="str">
         <v/>
       </c>
-      <c r="K4" t="str">
+      <c r="K5" t="str">
         <v/>
       </c>
-      <c r="L4" t="str">
+      <c r="L5" t="str">
         <v/>
       </c>
-      <c r="M4" t="str">
+      <c r="M5" t="str">
         <v/>
       </c>
-      <c r="N4" t="str">
+      <c r="N5" t="str">
         <v>Capacity  Model</v>
       </c>
-      <c r="O4" t="str">
+      <c r="O5" t="str">
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
+    <row r="7">
+      <c r="A7" t="str">
         <v/>
       </c>
-      <c r="B6" t="str">
+      <c r="B7" t="str">
         <v xml:space="preserve">SLA </v>
       </c>
-      <c r="C6" t="str">
+      <c r="C7" t="str">
         <v/>
       </c>
-      <c r="D6" t="str">
+      <c r="D7" t="str">
         <v>Resource Model</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E7" t="str">
         <v/>
       </c>
-      <c r="F6" t="str">
+      <c r="F7" t="str">
         <v/>
       </c>
-      <c r="G6" t="str">
+      <c r="G7" t="str">
         <v/>
       </c>
-      <c r="H6" t="str">
+      <c r="H7" t="str">
         <v/>
       </c>
-      <c r="I6" t="str">
+      <c r="I7" t="str">
         <v/>
       </c>
-      <c r="J6" t="str">
+      <c r="J7" t="str">
         <v>Resource Distribution Model &amp; HA</v>
       </c>
-      <c r="K6" t="str">
+      <c r="K7" t="str">
         <v/>
       </c>
-      <c r="L6" t="str">
+      <c r="L7" t="str">
         <v/>
       </c>
-      <c r="M6" t="str">
+      <c r="M7" t="str">
         <v/>
       </c>
-      <c r="N6" t="str">
+      <c r="N7" t="str">
         <v>Capacity Model</v>
       </c>
-      <c r="O6" t="str">
+      <c r="O7" t="str">
         <v/>
       </c>
-      <c r="P6" t="str">
+      <c r="P7" t="str">
         <v/>
       </c>
-      <c r="Q6" t="str">
+      <c r="Q7" t="str">
         <v>Release Method</v>
       </c>
-      <c r="R6" t="str">
+      <c r="R7" t="str">
         <v/>
       </c>
-      <c r="S6" t="str">
+      <c r="S7" t="str">
         <v/>
       </c>
-      <c r="T6" t="str">
+      <c r="T7" t="str">
         <v>Release Configuration  &amp; Artifacts</v>
       </c>
-      <c r="U6" t="str">
+      <c r="U7" t="str">
         <v/>
       </c>
-      <c r="V6" t="str">
+      <c r="V7" t="str">
         <v/>
       </c>
-      <c r="W6" t="str">
+      <c r="W7" t="str">
         <v/>
       </c>
-      <c r="X6" t="str">
+      <c r="X7" t="str">
         <v>Use for and Method &amp; store</v>
       </c>
-      <c r="Y6" t="str">
+      <c r="Y7" t="str">
         <v/>
       </c>
-      <c r="Z6" t="str">
+      <c r="Z7" t="str">
         <v/>
       </c>
-      <c r="AA6" t="str">
+      <c r="AA7" t="str">
         <v>Full</v>
       </c>
-      <c r="AB6" t="str">
+      <c r="AB7" t="str">
         <v/>
       </c>
-      <c r="AC6" t="str">
+      <c r="AC7" t="str">
         <v>Incremental (log)</v>
       </c>
-      <c r="AD6" t="str">
+      <c r="AD7" t="str">
         <v/>
       </c>
-      <c r="AE6" t="str">
+      <c r="AE7" t="str">
         <v>Fail-over/Fail-Back (recover full capacity)</v>
       </c>
-      <c r="AF6" t="str">
+      <c r="AF7" t="str">
         <v/>
       </c>
-      <c r="AG6" t="str">
+      <c r="AG7" t="str">
         <v/>
       </c>
-      <c r="AH6" t="str">
+      <c r="AH7" t="str">
         <v/>
       </c>
-      <c r="AI6" t="str">
+      <c r="AI7" t="str">
         <v>Operation Model</v>
       </c>
-      <c r="AJ6" t="str">
+      <c r="AJ7" t="str">
         <v/>
       </c>
-      <c r="AK6" t="str">
+      <c r="AK7" t="str">
         <v>Cost Model</v>
       </c>
-      <c r="AL6" t="str">
+      <c r="AL7" t="str">
         <v/>
       </c>
     </row>
-    <row r="7" xml:space="preserve">
-      <c r="A7" t="str">
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
         <v>ENV</v>
       </c>
-      <c r="B7" t="str" xml:space="preserve">
+      <c r="B8" t="str" xml:space="preserve">
         <v xml:space="preserve">SLA
 Value</v>
       </c>
-      <c r="C7" t="str" xml:space="preserve">
+      <c r="C8" t="str" xml:space="preserve">
         <v xml:space="preserve">SLA
 Class</v>
       </c>
-      <c r="D7" t="str" xml:space="preserve">
+      <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">Proposal
  Modules</v>
       </c>
-      <c r="E7" t="str">
+      <c r="E8" t="str">
         <v>Hosting Model</v>
       </c>
-      <c r="F7" t="str" xml:space="preserve">
+      <c r="F8" t="str" xml:space="preserve">
         <v xml:space="preserve">Hosting 
 Provider</v>
       </c>
-      <c r="G7" t="str" xml:space="preserve">
+      <c r="G8" t="str" xml:space="preserve">
         <v xml:space="preserve">Technical Model
 Module</v>
       </c>
-      <c r="H7" t="str" xml:space="preserve">
+      <c r="H8" t="str" xml:space="preserve">
         <v xml:space="preserve"> Service  Resource 
 Vendor Name (Relations)</v>
       </c>
-      <c r="I7" t="str" xml:space="preserve">
+      <c r="I8" t="str" xml:space="preserve">
         <v xml:space="preserve">Service Resources 
 Implementation</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J8" t="str">
         <v># instances</v>
       </c>
-      <c r="K7" t="str">
+      <c r="K8" t="str">
         <v>Region/Zone Distribution</v>
       </c>
-      <c r="L7" t="str">
+      <c r="L8" t="str">
         <v>Distribution Method</v>
       </c>
-      <c r="M7" t="str" xml:space="preserve">
+      <c r="M8" t="str" xml:space="preserve">
         <v xml:space="preserve">Resource Role
 Distribution</v>
       </c>
-      <c r="N7" t="str" xml:space="preserve">
+      <c r="N8" t="str" xml:space="preserve">
         <v xml:space="preserve">Capacity
 Class</v>
       </c>
-      <c r="O7" t="str">
+      <c r="O8" t="str">
         <v>Method</v>
       </c>
-      <c r="P7" t="str">
+      <c r="P8" t="str">
         <v>Outages</v>
       </c>
-      <c r="Q7" t="str" xml:space="preserve">
+      <c r="Q8" t="str" xml:space="preserve">
         <v xml:space="preserve">Release
 Class</v>
       </c>
-      <c r="R7" t="str">
+      <c r="R8" t="str">
         <v>Method</v>
       </c>
-      <c r="S7" t="str">
+      <c r="S8" t="str">
         <v>Outages</v>
       </c>
-      <c r="T7" t="str" xml:space="preserve">
+      <c r="T8" t="str" xml:space="preserve">
         <v xml:space="preserve">Configuration
 Specification</v>
       </c>
-      <c r="U7" t="str" xml:space="preserve">
+      <c r="U8" t="str" xml:space="preserve">
         <v xml:space="preserve">Configuration
 Version</v>
       </c>
-      <c r="V7" t="str" xml:space="preserve">
+      <c r="V8" t="str" xml:space="preserve">
         <v xml:space="preserve">Deploy
 Artifact
 </v>
       </c>
-      <c r="W7" t="str" xml:space="preserve">
+      <c r="W8" t="str" xml:space="preserve">
         <v xml:space="preserve">Artifact 
 Registry</v>
       </c>
-      <c r="X7" t="str">
+      <c r="X8" t="str">
         <v>Use for</v>
       </c>
-      <c r="Y7" t="str">
+      <c r="Y8" t="str">
         <v>Method</v>
       </c>
-      <c r="Z7" t="str">
+      <c r="Z8" t="str">
         <v>Store</v>
       </c>
-      <c r="AA7" t="str">
+      <c r="AA8" t="str">
         <v>Freq.</v>
       </c>
-      <c r="AB7" t="str">
+      <c r="AB8" t="str">
         <v>Retention</v>
       </c>
-      <c r="AC7" t="str">
+      <c r="AC8" t="str">
         <v>Freq.</v>
       </c>
-      <c r="AD7" t="str">
+      <c r="AD8" t="str">
         <v>Retention</v>
       </c>
-      <c r="AE7" t="str" xml:space="preserve">
+      <c r="AE8" t="str" xml:space="preserve">
         <v xml:space="preserve">Recovery 
 Class</v>
       </c>
-      <c r="AF7" t="str">
+      <c r="AF8" t="str">
         <v>Method</v>
       </c>
-      <c r="AG7" t="str">
+      <c r="AG8" t="str">
         <v>RTO</v>
       </c>
-      <c r="AH7" t="str">
+      <c r="AH8" t="str">
         <v>RPO</v>
       </c>
-      <c r="AI7" t="str">
+      <c r="AI8" t="str">
         <v>Operated By</v>
       </c>
-      <c r="AJ7" t="str" xml:space="preserve">
+      <c r="AJ8" t="str" xml:space="preserve">
         <v xml:space="preserve">Operation other Activities
 (which  W3 activities)</v>
       </c>
-      <c r="AK7" t="str">
+      <c r="AK8" t="str">
         <v>Model</v>
       </c>
-      <c r="AL7" t="str">
+      <c r="AL8" t="str">
         <v>Details</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B8" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C8" t="str">
-        <v>HA</v>
-      </c>
-      <c r="D8" t="str">
-        <v>INFRASTRUCTURE</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Seeweb S.r.l.</v>
-      </c>
-      <c r="I8" t="str">
-        <v>Virtualization Platform - ProxMox</v>
-      </c>
-      <c r="J8" t="str">
-        <v>1 Cluster Multinodo</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Seeweb Italy (DC1)</v>
-      </c>
-      <c r="L8" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M8" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N8" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O8" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P8" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q8" t="str">
-        <v>Ops - Manual</v>
-      </c>
-      <c r="R8" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S8" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T8" t="str">
-        <v>File (TXT)</v>
-      </c>
-      <c r="U8" t="str">
-        <v>Proxmox VE 8.x</v>
-      </c>
-      <c r="V8" t="str">
-        <v>VMI (virtual Machine Image) - KVM</v>
-      </c>
-      <c r="W8" t="str">
-        <v>Private Others Registry</v>
-      </c>
-      <c r="X8" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y8" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z8" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA8" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB8" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC8" t="str">
-        <v>1 min</v>
-      </c>
-      <c r="AD8" t="str">
-        <v>1 week</v>
-      </c>
-      <c r="AE8" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF8" t="str">
-        <v>Automated By App</v>
-      </c>
-      <c r="AG8" t="str">
-        <v>Minutes (1-5)</v>
-      </c>
-      <c r="AH8" t="str">
-        <v>Minutes (1-5)</v>
-      </c>
-      <c r="AI8" t="str">
-        <v>HW/SW vendor</v>
-      </c>
-      <c r="AJ8" t="str">
-        <v>Cluster Management</v>
-      </c>
-      <c r="AK8" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL8" t="str">
-        <v>Seeweb Multinodo Contract</v>
       </c>
     </row>
     <row r="9">
@@ -6383,10 +6129,10 @@
         <v>PROD</v>
       </c>
       <c r="B9" t="str">
-        <v>99,5%</v>
+        <v>99,9%</v>
       </c>
       <c r="C9" t="str">
-        <v>HA-</v>
+        <v>HA</v>
       </c>
       <c r="D9" t="str">
         <v>INFRASTRUCTURE</v>
@@ -6398,19 +6144,19 @@
         <v>Vendor Private</v>
       </c>
       <c r="G9" t="str">
-        <v>HW Appliance</v>
+        <v>Full IaaS</v>
       </c>
       <c r="H9" t="str">
-        <v>Seeweb S.r.l. (Fortinet)</v>
+        <v>Seeweb S.r.l. - Proxmox VE Cluster</v>
       </c>
       <c r="I9" t="str">
-        <v>HW Appliance - FortiGate NGFW</v>
-      </c>
-      <c r="J9" t="str">
-        <v>1 (Single)</v>
+        <v>Virtualization Platform - ProxMox</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
       </c>
       <c r="K9" t="str">
-        <v>Seeweb Italy (DC1)</v>
+        <v>Cloud-Single-zone</v>
       </c>
       <c r="L9" t="str">
         <v>Resources - SW configuration</v>
@@ -6419,10 +6165,10 @@
         <v>Active</v>
       </c>
       <c r="N9" t="str">
-        <v>Fixed capacity</v>
+        <v>Ops Manual</v>
       </c>
       <c r="O9" t="str">
-        <v>Do not scale - Fixed capacity</v>
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P9" t="str">
         <v>No outages</v>
@@ -6437,13 +6183,13 @@
         <v>No outages</v>
       </c>
       <c r="T9" t="str">
-        <v>File (TXT)</v>
+        <v>Configuration File (TXT)</v>
       </c>
       <c r="U9" t="str">
-        <v>FortiOS 7.x</v>
+        <v>Vendor Versioning</v>
       </c>
       <c r="V9" t="str">
-        <v>SW Bins</v>
+        <v>VMI (Virtual Machine Image) - KVM</v>
       </c>
       <c r="W9" t="str">
         <v>Private Others Registry</v>
@@ -6464,34 +6210,34 @@
         <v>1 month</v>
       </c>
       <c r="AC9" t="str">
-        <v>N/A</v>
+        <v>1 min</v>
       </c>
       <c r="AD9" t="str">
-        <v>N/A</v>
+        <v>1 week</v>
       </c>
       <c r="AE9" t="str">
-        <v xml:space="preserve">Local Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF9" t="str">
-        <v>Manual By Operation</v>
+        <v>Automated By App</v>
       </c>
       <c r="AG9" t="str">
-        <v>Hour (1-5)</v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AH9" t="str">
-        <v>Hour (1-5)</v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AI9" t="str">
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ9" t="str">
-        <v>Security Management</v>
+        <v>Cluster Management, VM Provisioning</v>
       </c>
       <c r="AK9" t="str">
-        <v>COTs SW License</v>
+        <v>Public Cloud Consumption</v>
       </c>
       <c r="AL9" t="str">
-        <v>Seeweb FortiGate Service</v>
+        <v>Seeweb Multinodo Contract</v>
       </c>
     </row>
     <row r="10">
@@ -6499,10 +6245,10 @@
         <v>PROD</v>
       </c>
       <c r="B10" t="str">
-        <v>99,9%</v>
+        <v>99,5%</v>
       </c>
       <c r="C10" t="str">
-        <v>HA</v>
+        <v>HA-</v>
       </c>
       <c r="D10" t="str">
         <v>INFRASTRUCTURE</v>
@@ -6514,31 +6260,31 @@
         <v>Vendor Private</v>
       </c>
       <c r="G10" t="str">
-        <v>Bare Metal</v>
+        <v>HW Appliance</v>
       </c>
       <c r="H10" t="str">
-        <v>Seeweb S.r.l.</v>
+        <v>Seeweb S.r.l. - Fortinet FortiGate</v>
       </c>
       <c r="I10" t="str">
-        <v>Bare Metal-Linux OS</v>
-      </c>
-      <c r="J10" t="str">
-        <v>1 (Dedicato)</v>
+        <v>HW Appliance - FortiGate NGFW</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
       </c>
       <c r="K10" t="str">
-        <v>Seeweb Italy (DC2 - DR)</v>
+        <v>Cloud-Single-zone</v>
       </c>
       <c r="L10" t="str">
-        <v>Resources - SW configuration</v>
+        <v>Resource - Manual Installation</v>
       </c>
       <c r="M10" t="str">
         <v>Active</v>
       </c>
       <c r="N10" t="str">
-        <v>Ops Manual</v>
+        <v>Fixed capacity</v>
       </c>
       <c r="O10" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+        <v>Do not scale - Fixed capacity</v>
       </c>
       <c r="P10" t="str">
         <v>No outages</v>
@@ -6553,16 +6299,16 @@
         <v>No outages</v>
       </c>
       <c r="T10" t="str">
-        <v>File (TXT)</v>
+        <v>Configuration File (TXT)</v>
       </c>
       <c r="U10" t="str">
-        <v>PBS 3.x</v>
+        <v>Vendor Versioning</v>
       </c>
       <c r="V10" t="str">
         <v>SW Bins</v>
       </c>
       <c r="W10" t="str">
-        <v>Object Store (SW bins)</v>
+        <v>Private Others Registry</v>
       </c>
       <c r="X10" t="str">
         <v>Resource Recovery</v>
@@ -6580,13 +6326,13 @@
         <v>1 month</v>
       </c>
       <c r="AC10" t="str">
-        <v>1 min</v>
+        <v>N/A</v>
       </c>
       <c r="AD10" t="str">
-        <v>1 week</v>
+        <v>N/A</v>
       </c>
       <c r="AE10" t="str">
-        <v xml:space="preserve">Region Resilent </v>
+        <v xml:space="preserve">Local Resilent </v>
       </c>
       <c r="AF10" t="str">
         <v>Manual By Operation</v>
@@ -6595,19 +6341,19 @@
         <v>Hour (1-5)</v>
       </c>
       <c r="AH10" t="str">
-        <v>Minutes (1-5)</v>
+        <v>Hour (1-5)</v>
       </c>
       <c r="AI10" t="str">
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ10" t="str">
-        <v>Backup &amp; DR</v>
+        <v>Security Policy, Threat Monitoring</v>
       </c>
       <c r="AK10" t="str">
-        <v>Public Cloud Consumption</v>
+        <v>COTs SW License</v>
       </c>
       <c r="AL10" t="str">
-        <v>Seeweb PBS Service</v>
+        <v>FortiCare via Seeweb</v>
       </c>
     </row>
     <row r="11">
@@ -6621,7 +6367,7 @@
         <v>HA</v>
       </c>
       <c r="D11" t="str">
-        <v>APPLICATION</v>
+        <v>INFRASTRUCTURE</v>
       </c>
       <c r="E11" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6630,19 +6376,19 @@
         <v>Vendor Private</v>
       </c>
       <c r="G11" t="str">
-        <v>Full IaaS</v>
+        <v>Bare Metal</v>
       </c>
       <c r="H11" t="str">
-        <v>Seeweb S.r.l.</v>
+        <v>Seeweb S.r.l. - Proxmox Backup Server</v>
       </c>
       <c r="I11" t="str">
-        <v>App (RunTime) - Linux native</v>
-      </c>
-      <c r="J11" t="str">
-        <v>1 VPC (Nginx + LB)</v>
+        <v>Bare Metal - PBS Dedicated</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
       </c>
       <c r="K11" t="str">
-        <v>Seeweb Italy (DC1)</v>
+        <v>Cloud-Single-zone</v>
       </c>
       <c r="L11" t="str">
         <v>Resources - SW configuration</v>
@@ -6660,7 +6406,7 @@
         <v>No outages</v>
       </c>
       <c r="Q11" t="str">
-        <v>Ops - Automated</v>
+        <v>Ops - Manual</v>
       </c>
       <c r="R11" t="str">
         <v>Ops Manual - direct Log-on resource</v>
@@ -6669,10 +6415,10 @@
         <v>No outages</v>
       </c>
       <c r="T11" t="str">
-        <v>File (Ansible playbook) - VM configuration</v>
+        <v>Configuration File (TXT)</v>
       </c>
       <c r="U11" t="str">
-        <v>Nginx 1.24 + W3Suite FE</v>
+        <v>Vendor Versioning</v>
       </c>
       <c r="V11" t="str">
         <v>SW Bins</v>
@@ -6705,25 +6451,25 @@
         <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF11" t="str">
-        <v>Automated By App</v>
+        <v>Manual By Operation</v>
       </c>
       <c r="AG11" t="str">
-        <v xml:space="preserve">Seconds </v>
+        <v>Hour (1-5)</v>
       </c>
       <c r="AH11" t="str">
-        <v>N/A</v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AI11" t="str">
-        <v>SW Integrator</v>
+        <v>HW/SW vendor</v>
       </c>
       <c r="AJ11" t="str">
-        <v>TLS, Routing, LB Config</v>
+        <v>Backup Storage, DR Recovery</v>
       </c>
       <c r="AK11" t="str">
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL11" t="str">
-        <v>Seeweb VPC</v>
+        <v>Seeweb PBS Service</v>
       </c>
     </row>
     <row r="12">
@@ -6749,16 +6495,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H12" t="str">
-        <v>Seeweb S.r.l.</v>
+        <v>Seeweb S.r.l. - W3Suite Frontend</v>
       </c>
       <c r="I12" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
-      <c r="J12" t="str">
-        <v>1 VPC (API+Redis+MCP)</v>
+      <c r="J12">
+        <v>1</v>
       </c>
       <c r="K12" t="str">
-        <v>Seeweb Italy (DC1)</v>
+        <v>Cloud-Single-zone</v>
       </c>
       <c r="L12" t="str">
         <v>Resources - SW configuration</v>
@@ -6779,16 +6525,16 @@
         <v>Ops - Automated</v>
       </c>
       <c r="R12" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
+        <v xml:space="preserve">Ops Automated (SW) - DevOps </v>
       </c>
       <c r="S12" t="str">
         <v>No outages</v>
       </c>
       <c r="T12" t="str">
-        <v>File (Ansible playbook) - VM configuration</v>
+        <v>Configuration File (YAML)</v>
       </c>
       <c r="U12" t="str">
-        <v>W3Suite API + Redis + MCP</v>
+        <v>W3 Git</v>
       </c>
       <c r="V12" t="str">
         <v>SW Bins</v>
@@ -6824,7 +6570,7 @@
         <v>Automated By App</v>
       </c>
       <c r="AG12" t="str">
-        <v>Minutes (1-5)</v>
+        <v xml:space="preserve">Seconds </v>
       </c>
       <c r="AH12" t="str">
         <v xml:space="preserve">Seconds </v>
@@ -6833,7 +6579,7 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ12" t="str">
-        <v>Deploy, API, AI Gateway</v>
+        <v>TLS, Routing, LB Config</v>
       </c>
       <c r="AK12" t="str">
         <v>Public Cloud Consumption</v>
@@ -6853,7 +6599,7 @@
         <v>HA</v>
       </c>
       <c r="D13" t="str">
-        <v>DATABASE</v>
+        <v>APPLICATION</v>
       </c>
       <c r="E13" t="str">
         <v>Not W3 Private datacenter</v>
@@ -6865,16 +6611,16 @@
         <v>Full IaaS</v>
       </c>
       <c r="H13" t="str">
-        <v>Seeweb S.r.l.</v>
+        <v>Seeweb S.r.l. - W3Suite Backend</v>
       </c>
       <c r="I13" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
-      <c r="J13" t="str">
-        <v>1 VPC (PostgreSQL Primary)</v>
+      <c r="J13">
+        <v>1</v>
       </c>
       <c r="K13" t="str">
-        <v>Seeweb Italy (DC1)</v>
+        <v>Cloud-Single-zone</v>
       </c>
       <c r="L13" t="str">
         <v>Resources - SW configuration</v>
@@ -6889,22 +6635,22 @@
         <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P13" t="str">
-        <v>Minutes (1-10)</v>
+        <v>No outages</v>
       </c>
       <c r="Q13" t="str">
-        <v>Ops - Manual</v>
+        <v>Ops - Automated</v>
       </c>
       <c r="R13" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
+        <v xml:space="preserve">Ops Automated (SW) - DevOps </v>
       </c>
       <c r="S13" t="str">
-        <v>Minutes (1-10)</v>
+        <v>No outages</v>
       </c>
       <c r="T13" t="str">
-        <v>File (TXT)</v>
+        <v>Configuration File (YAML)</v>
       </c>
       <c r="U13" t="str">
-        <v>PostgreSQL 15.x</v>
+        <v>W3 Git</v>
       </c>
       <c r="V13" t="str">
         <v>SW Bins</v>
@@ -6913,7 +6659,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X13" t="str">
-        <v>Resource: Release and Recovery</v>
+        <v>Resource Recovery</v>
       </c>
       <c r="Y13" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -6949,7 +6695,7 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ13" t="str">
-        <v>Backup, Tuning, PITR</v>
+        <v>Deploy, API, AI Gateway, Cache</v>
       </c>
       <c r="AK13" t="str">
         <v>Public Cloud Consumption</v>
@@ -6966,7 +6712,7 @@
         <v>99,9%</v>
       </c>
       <c r="C14" t="str">
-        <v>HA</v>
+        <v>HA+</v>
       </c>
       <c r="D14" t="str">
         <v>DATABASE</v>
@@ -6981,22 +6727,22 @@
         <v>Full IaaS</v>
       </c>
       <c r="H14" t="str">
-        <v>Seeweb S.r.l.</v>
+        <v>Seeweb S.r.l. - PostgreSQL Primary</v>
       </c>
       <c r="I14" t="str">
         <v>App (RunTime) - Linux native</v>
       </c>
-      <c r="J14" t="str">
-        <v>1 VPC (PostgreSQL Replica)</v>
+      <c r="J14">
+        <v>1</v>
       </c>
       <c r="K14" t="str">
-        <v>Seeweb Italy (DC1)</v>
+        <v>Cloud-Single-zone</v>
       </c>
       <c r="L14" t="str">
         <v>Resources - SW configuration</v>
       </c>
       <c r="M14" t="str">
-        <v>Standby</v>
+        <v>Active</v>
       </c>
       <c r="N14" t="str">
         <v>Ops Manual</v>
@@ -7005,7 +6751,7 @@
         <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P14" t="str">
-        <v>No outages</v>
+        <v>Minutes (1-10)</v>
       </c>
       <c r="Q14" t="str">
         <v>Ops - Manual</v>
@@ -7014,13 +6760,13 @@
         <v>Ops Manual - direct Log-on resource</v>
       </c>
       <c r="S14" t="str">
-        <v>No outages</v>
+        <v>Minutes (1-10)</v>
       </c>
       <c r="T14" t="str">
-        <v>File (TXT)</v>
+        <v>Configuration File (TXT)</v>
       </c>
       <c r="U14" t="str">
-        <v>PostgreSQL 15.x</v>
+        <v>Vendor Versioning</v>
       </c>
       <c r="V14" t="str">
         <v>SW Bins</v>
@@ -7029,7 +6775,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X14" t="str">
-        <v>Resource Recovery</v>
+        <v>Resource: Release and Recovery</v>
       </c>
       <c r="Y14" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -7056,7 +6802,7 @@
         <v>Automated By App</v>
       </c>
       <c r="AG14" t="str">
-        <v xml:space="preserve">Seconds </v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AH14" t="str">
         <v xml:space="preserve">Seconds </v>
@@ -7065,7 +6811,7 @@
         <v>SW Integrator</v>
       </c>
       <c r="AJ14" t="str">
-        <v>Streaming Replication</v>
+        <v>Backup, Tuning, PITR, WAL</v>
       </c>
       <c r="AK14" t="str">
         <v>Public Cloud Consumption</v>
@@ -7074,9 +6820,380 @@
         <v>Seeweb VPC</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B15" t="str">
+        <v>99,9%</v>
+      </c>
+      <c r="C15" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D15" t="str">
+        <v>DATABASE</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Full IaaS</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Seeweb S.r.l. - PostgreSQL Replica</v>
+      </c>
+      <c r="I15" t="str">
+        <v>App (RunTime) - Linux native</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Cloud-Single-zone</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Resources - SW configuration</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Standby</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Ops Manual</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+      </c>
+      <c r="P15" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>Ops - Manual</v>
+      </c>
+      <c r="R15" t="str">
+        <v>Ops Manual - direct Log-on resource</v>
+      </c>
+      <c r="S15" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="T15" t="str">
+        <v>Configuration File (TXT)</v>
+      </c>
+      <c r="U15" t="str">
+        <v>Vendor Versioning</v>
+      </c>
+      <c r="V15" t="str">
+        <v>SW Bins</v>
+      </c>
+      <c r="W15" t="str">
+        <v>Object Store (SW bins)</v>
+      </c>
+      <c r="X15" t="str">
+        <v>Resource Recovery</v>
+      </c>
+      <c r="Y15" t="str">
+        <v>On-Premise SW/Appliance</v>
+      </c>
+      <c r="Z15" t="str">
+        <v>On-premise Store (Appliance)</v>
+      </c>
+      <c r="AA15" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="AB15" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC15" t="str">
+        <v>1 min</v>
+      </c>
+      <c r="AD15" t="str">
+        <v>1 week</v>
+      </c>
+      <c r="AE15" t="str">
+        <v xml:space="preserve">Region Resilent </v>
+      </c>
+      <c r="AF15" t="str">
+        <v>Automated By App</v>
+      </c>
+      <c r="AG15" t="str">
+        <v xml:space="preserve">Seconds </v>
+      </c>
+      <c r="AH15" t="str">
+        <v xml:space="preserve">Seconds </v>
+      </c>
+      <c r="AI15" t="str">
+        <v>SW Integrator</v>
+      </c>
+      <c r="AJ15" t="str">
+        <v>Streaming Replication, Failover</v>
+      </c>
+      <c r="AK15" t="str">
+        <v>Public Cloud Consumption</v>
+      </c>
+      <c r="AL15" t="str">
+        <v>Seeweb VPC</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A4:AL14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AL15"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A2:G15"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="25.83203125" customWidth="1"/>
+    <col min="7" max="7" width="25.83203125" customWidth="1"/>
+    <col min="8" max="8" width="25.83203125" customWidth="1"/>
+    <col min="9" max="9" width="25.83203125" customWidth="1"/>
+    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Public Cloud Zones or W3 Sites</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Field Definition &amp; Values 
+Module of solution</v>
+      </c>
+      <c r="B3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Field Definition &amp; Values 
+Resource of module</v>
+      </c>
+      <c r="C3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Field Definition &amp; Values
+Resource component</v>
+      </c>
+      <c r="D3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Field Definition &amp; Values
+Sites List</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>Module</v>
+      </c>
+      <c r="B7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Service
+Resources</v>
+      </c>
+      <c r="C7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Resource 
+Component (if needed)</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Region (Zone/site)</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Zone/site</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Zone/site</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Zone/site</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>Seeweb Italy DC1</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Seeweb Italy DC2</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>INFRASTRUCTURE</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Proxmox VE Cluster</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Multinodo Cluster</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Seeweb DC1 (Primary)</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>INFRASTRUCTURE</v>
+      </c>
+      <c r="B10" t="str">
+        <v>FortiGate NGFW</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Single Appliance</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Seeweb DC1</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>INFRASTRUCTURE</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Proxmox Backup Server</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Dedicated Server</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v>Seeweb DC2 (DR)</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>APPLICATION</v>
+      </c>
+      <c r="B12" t="str">
+        <v>W3Suite Frontend</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Nginx + LB</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Seeweb DC1</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>APPLICATION</v>
+      </c>
+      <c r="B13" t="str">
+        <v>W3Suite Backend</v>
+      </c>
+      <c r="C13" t="str">
+        <v>API + Redis + MCP</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Seeweb DC1</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>DATABASE</v>
+      </c>
+      <c r="B14" t="str">
+        <v>PostgreSQL Primary</v>
+      </c>
+      <c r="C14" t="str">
+        <v>DB Primary</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Seeweb DC1</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>DATABASE</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PostgreSQL Replica</v>
+      </c>
+      <c r="C15" t="str">
+        <v>DB Standby</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Seeweb DC1</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A2:G15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update resource model documentation for cloud and hardware configurations
Update various versions of the Excel resource model documentation to reflect accurate cloud and hardware deployment configurations, including multi-region distribution for clusters and specific handling for hardware appliances.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c5a1ca68-c987-4ef1-9a95-626de70f72f4
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
+++ b/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
@@ -5778,6 +5778,1175 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AL15"/>
   <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="24.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="24.83203125" customWidth="1"/>
+    <col min="17" max="17" width="24.83203125" customWidth="1"/>
+    <col min="18" max="18" width="24.83203125" customWidth="1"/>
+    <col min="19" max="19" width="24.83203125" customWidth="1"/>
+    <col min="20" max="20" width="24.83203125" customWidth="1"/>
+    <col min="21" max="21" width="24.83203125" customWidth="1"/>
+    <col min="22" max="22" width="24.83203125" customWidth="1"/>
+    <col min="23" max="23" width="24.83203125" customWidth="1"/>
+    <col min="24" max="24" width="24.83203125" customWidth="1"/>
+    <col min="25" max="25" width="24.83203125" customWidth="1"/>
+    <col min="26" max="26" width="24.83203125" customWidth="1"/>
+    <col min="27" max="27" width="24.83203125" customWidth="1"/>
+    <col min="28" max="28" width="24.83203125" customWidth="1"/>
+    <col min="29" max="29" width="24.83203125" customWidth="1"/>
+    <col min="30" max="30" width="24.83203125" customWidth="1"/>
+    <col min="31" max="31" width="24.83203125" customWidth="1"/>
+    <col min="32" max="32" width="24.83203125" customWidth="1"/>
+    <col min="33" max="33" width="24.83203125" customWidth="1"/>
+    <col min="34" max="34" width="24.83203125" customWidth="1"/>
+    <col min="35" max="35" width="24.83203125" customWidth="1"/>
+    <col min="36" max="36" width="24.83203125" customWidth="1"/>
+    <col min="37" max="37" width="24.83203125" customWidth="1"/>
+    <col min="38" max="38" width="24.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>W3Suite - Service Resource Model - Seeweb Infrastructure</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Environment</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SLA Model &amp; Resource Model</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v>Capacity  Model</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v xml:space="preserve">SLA </v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Resource Model</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v>Resource Distribution Model &amp; HA</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v>Capacity Model</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>Release Method</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v>Release Configuration  &amp; Artifacts</v>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v>Use for and Method &amp; store</v>
+      </c>
+      <c r="Y7" t="str">
+        <v/>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
+      </c>
+      <c r="AA7" t="str">
+        <v>Full</v>
+      </c>
+      <c r="AB7" t="str">
+        <v/>
+      </c>
+      <c r="AC7" t="str">
+        <v>Incremental (log)</v>
+      </c>
+      <c r="AD7" t="str">
+        <v/>
+      </c>
+      <c r="AE7" t="str">
+        <v>Fail-over/Fail-Back (recover full capacity)</v>
+      </c>
+      <c r="AF7" t="str">
+        <v/>
+      </c>
+      <c r="AG7" t="str">
+        <v/>
+      </c>
+      <c r="AH7" t="str">
+        <v/>
+      </c>
+      <c r="AI7" t="str">
+        <v>Operation Model</v>
+      </c>
+      <c r="AJ7" t="str">
+        <v/>
+      </c>
+      <c r="AK7" t="str">
+        <v>Cost Model</v>
+      </c>
+      <c r="AL7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>ENV</v>
+      </c>
+      <c r="B8" t="str" xml:space="preserve">
+        <v xml:space="preserve">SLA
+Value</v>
+      </c>
+      <c r="C8" t="str" xml:space="preserve">
+        <v xml:space="preserve">SLA
+Class</v>
+      </c>
+      <c r="D8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Proposal
+ Modules</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Hosting Model</v>
+      </c>
+      <c r="F8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hosting 
+Provider</v>
+      </c>
+      <c r="G8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Technical Model
+Module</v>
+      </c>
+      <c r="H8" t="str" xml:space="preserve">
+        <v xml:space="preserve"> Service  Resource 
+Vendor Name (Relations)</v>
+      </c>
+      <c r="I8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Service Resources 
+Implementation</v>
+      </c>
+      <c r="J8" t="str">
+        <v># instances</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Region/Zone Distribution</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Distribution Method</v>
+      </c>
+      <c r="M8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Resource Role
+Distribution</v>
+      </c>
+      <c r="N8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Capacity
+Class</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Method</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Outages</v>
+      </c>
+      <c r="Q8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Release
+Class</v>
+      </c>
+      <c r="R8" t="str">
+        <v>Method</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Outages</v>
+      </c>
+      <c r="T8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Configuration
+Specification</v>
+      </c>
+      <c r="U8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Configuration
+Version</v>
+      </c>
+      <c r="V8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Deploy
+Artifact
+</v>
+      </c>
+      <c r="W8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Artifact 
+Registry</v>
+      </c>
+      <c r="X8" t="str">
+        <v>Use for</v>
+      </c>
+      <c r="Y8" t="str">
+        <v>Method</v>
+      </c>
+      <c r="Z8" t="str">
+        <v>Store</v>
+      </c>
+      <c r="AA8" t="str">
+        <v>Freq.</v>
+      </c>
+      <c r="AB8" t="str">
+        <v>Retention</v>
+      </c>
+      <c r="AC8" t="str">
+        <v>Freq.</v>
+      </c>
+      <c r="AD8" t="str">
+        <v>Retention</v>
+      </c>
+      <c r="AE8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Recovery 
+Class</v>
+      </c>
+      <c r="AF8" t="str">
+        <v>Method</v>
+      </c>
+      <c r="AG8" t="str">
+        <v>RTO</v>
+      </c>
+      <c r="AH8" t="str">
+        <v>RPO</v>
+      </c>
+      <c r="AI8" t="str">
+        <v>Operated By</v>
+      </c>
+      <c r="AJ8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Operation other Activities
+(which  W3 activities)</v>
+      </c>
+      <c r="AK8" t="str">
+        <v>Model</v>
+      </c>
+      <c r="AL8" t="str">
+        <v>Details</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B9" t="str">
+        <v>99,9%</v>
+      </c>
+      <c r="C9" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D9" t="str">
+        <v>INFRASTRUCTURE</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Full IaaS</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Seeweb S.r.l. - Proxmox VE Cluster</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Virtualization Platform - ProxMox</v>
+      </c>
+      <c r="J9" t="str">
+        <v>3+ nodi</v>
+      </c>
+      <c r="K9" t="str">
+        <v xml:space="preserve">Cloud-Multi-region </v>
+      </c>
+      <c r="L9" t="str">
+        <v>Resources - SW configuration</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Active</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Ops Manual</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+      </c>
+      <c r="P9" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>Ops - Manual</v>
+      </c>
+      <c r="R9" t="str">
+        <v>Ops Manual - direct Log-on resource</v>
+      </c>
+      <c r="S9" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="T9" t="str">
+        <v>Configuration File (TXT)</v>
+      </c>
+      <c r="U9" t="str">
+        <v>Vendor Versioning</v>
+      </c>
+      <c r="V9" t="str">
+        <v>VMI (Virtual Machine Image) - KVM</v>
+      </c>
+      <c r="W9" t="str">
+        <v>Private Others Registry</v>
+      </c>
+      <c r="X9" t="str">
+        <v>Resource Recovery</v>
+      </c>
+      <c r="Y9" t="str">
+        <v>On-Premise SW/Appliance</v>
+      </c>
+      <c r="Z9" t="str">
+        <v>On-premise Store (Appliance)</v>
+      </c>
+      <c r="AA9" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="AB9" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC9" t="str">
+        <v>1 min</v>
+      </c>
+      <c r="AD9" t="str">
+        <v>1 week</v>
+      </c>
+      <c r="AE9" t="str">
+        <v xml:space="preserve">Region Resilent </v>
+      </c>
+      <c r="AF9" t="str">
+        <v>Automated By App</v>
+      </c>
+      <c r="AG9" t="str">
+        <v>Minutes (1-5)</v>
+      </c>
+      <c r="AH9" t="str">
+        <v>Minutes (1-5)</v>
+      </c>
+      <c r="AI9" t="str">
+        <v>HW/SW vendor</v>
+      </c>
+      <c r="AJ9" t="str">
+        <v>Cluster Management, VM Provisioning, HA</v>
+      </c>
+      <c r="AK9" t="str">
+        <v>Public Cloud Consumption</v>
+      </c>
+      <c r="AL9" t="str">
+        <v>Seeweb Multinodo Contract</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B10" t="str">
+        <v>99,5%</v>
+      </c>
+      <c r="C10" t="str">
+        <v>HA-</v>
+      </c>
+      <c r="D10" t="str">
+        <v>INFRASTRUCTURE</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G10" t="str">
+        <v>HW Appliance</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Seeweb S.r.l. - Fortinet FortiGate</v>
+      </c>
+      <c r="I10" t="str">
+        <v>HW Appliance - FortiGate NGFW</v>
+      </c>
+      <c r="J10" t="str">
+        <v>1 (Single)</v>
+      </c>
+      <c r="K10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Resource - Manual Installation</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Active</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Fixed capacity</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Do not scale - Fixed capacity</v>
+      </c>
+      <c r="P10" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>Ops - Manual</v>
+      </c>
+      <c r="R10" t="str">
+        <v>Ops Manual - direct Log-on resource</v>
+      </c>
+      <c r="S10" t="str">
+        <v>Hours (1-5)</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Configuration File (TXT)</v>
+      </c>
+      <c r="U10" t="str">
+        <v>Vendor Versioning</v>
+      </c>
+      <c r="V10" t="str">
+        <v>SW Bins</v>
+      </c>
+      <c r="W10" t="str">
+        <v>Private Others Registry</v>
+      </c>
+      <c r="X10" t="str">
+        <v>Resource Recovery</v>
+      </c>
+      <c r="Y10" t="str">
+        <v>On-Premise SW/Appliance</v>
+      </c>
+      <c r="Z10" t="str">
+        <v>On-premise Store (Appliance)</v>
+      </c>
+      <c r="AA10" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="AB10" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AD10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AE10" t="str">
+        <v xml:space="preserve">Local Resilent </v>
+      </c>
+      <c r="AF10" t="str">
+        <v>Manual By Operation</v>
+      </c>
+      <c r="AG10" t="str">
+        <v>Hour (1-5)</v>
+      </c>
+      <c r="AH10" t="str">
+        <v>Hour (1-5)</v>
+      </c>
+      <c r="AI10" t="str">
+        <v>HW/SW vendor</v>
+      </c>
+      <c r="AJ10" t="str">
+        <v>Security Policy, Threat Monitoring, FW Rules</v>
+      </c>
+      <c r="AK10" t="str">
+        <v>(on-premise) HW Buy &amp; Support</v>
+      </c>
+      <c r="AL10" t="str">
+        <v>FortiGate HW + FortiCare Support</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B11" t="str">
+        <v>99,9%</v>
+      </c>
+      <c r="C11" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D11" t="str">
+        <v>INFRASTRUCTURE</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Bare Metal</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Seeweb S.r.l. - Proxmox Backup Server</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Bare Metal - PBS Dedicated</v>
+      </c>
+      <c r="J11" t="str">
+        <v>1 (Dedicato)</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Cloud-Single-zone</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Resources - SW configuration</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Active</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Ops Manual</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+      </c>
+      <c r="P11" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>Ops - Manual</v>
+      </c>
+      <c r="R11" t="str">
+        <v>Ops Manual - direct Log-on resource</v>
+      </c>
+      <c r="S11" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="T11" t="str">
+        <v>Configuration File (TXT)</v>
+      </c>
+      <c r="U11" t="str">
+        <v>Vendor Versioning</v>
+      </c>
+      <c r="V11" t="str">
+        <v>SW Bins</v>
+      </c>
+      <c r="W11" t="str">
+        <v>Object Store (SW bins)</v>
+      </c>
+      <c r="X11" t="str">
+        <v>Resource Recovery</v>
+      </c>
+      <c r="Y11" t="str">
+        <v>On-Premise SW/Appliance</v>
+      </c>
+      <c r="Z11" t="str">
+        <v>On-premise Store (Appliance)</v>
+      </c>
+      <c r="AA11" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="AB11" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC11" t="str">
+        <v>1 min</v>
+      </c>
+      <c r="AD11" t="str">
+        <v>1 week</v>
+      </c>
+      <c r="AE11" t="str">
+        <v xml:space="preserve">Region Resilent </v>
+      </c>
+      <c r="AF11" t="str">
+        <v>Manual By Operation</v>
+      </c>
+      <c r="AG11" t="str">
+        <v>Hour (1-5)</v>
+      </c>
+      <c r="AH11" t="str">
+        <v>Minutes (1-5)</v>
+      </c>
+      <c r="AI11" t="str">
+        <v>HW/SW vendor</v>
+      </c>
+      <c r="AJ11" t="str">
+        <v>Backup Storage, DR Recovery, Retention</v>
+      </c>
+      <c r="AK11" t="str">
+        <v>Public Cloud Consumption</v>
+      </c>
+      <c r="AL11" t="str">
+        <v>Seeweb PBS Service</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B12" t="str">
+        <v>99,9%</v>
+      </c>
+      <c r="C12" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D12" t="str">
+        <v>APPLICATION</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Full IaaS</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Seeweb S.r.l. - W3Suite Frontend</v>
+      </c>
+      <c r="I12" t="str">
+        <v>App (RunTime) - Linux native</v>
+      </c>
+      <c r="J12" t="str">
+        <v>1 VPC</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Cloud-Single-zone</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Resources - SW configuration</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Active</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Ops Manual</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+      </c>
+      <c r="P12" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>Ops - Automated</v>
+      </c>
+      <c r="R12" t="str">
+        <v xml:space="preserve">Ops Automated (SW) - DevOps </v>
+      </c>
+      <c r="S12" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="T12" t="str">
+        <v>Configuration File (YAML)</v>
+      </c>
+      <c r="U12" t="str">
+        <v>W3 Git</v>
+      </c>
+      <c r="V12" t="str">
+        <v>SW Bins</v>
+      </c>
+      <c r="W12" t="str">
+        <v>Object Store (SW bins)</v>
+      </c>
+      <c r="X12" t="str">
+        <v>Resource Recovery</v>
+      </c>
+      <c r="Y12" t="str">
+        <v>On-Premise SW/Appliance</v>
+      </c>
+      <c r="Z12" t="str">
+        <v>On-premise Store (Appliance)</v>
+      </c>
+      <c r="AA12" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="AB12" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC12" t="str">
+        <v>1 min</v>
+      </c>
+      <c r="AD12" t="str">
+        <v>1 week</v>
+      </c>
+      <c r="AE12" t="str">
+        <v xml:space="preserve">Region Resilent </v>
+      </c>
+      <c r="AF12" t="str">
+        <v>Automated By App</v>
+      </c>
+      <c r="AG12" t="str">
+        <v xml:space="preserve">Seconds </v>
+      </c>
+      <c r="AH12" t="str">
+        <v xml:space="preserve">Seconds </v>
+      </c>
+      <c r="AI12" t="str">
+        <v>SW Integrator</v>
+      </c>
+      <c r="AJ12" t="str">
+        <v>TLS, Routing, LB Config, CDN</v>
+      </c>
+      <c r="AK12" t="str">
+        <v>Public Cloud Consumption</v>
+      </c>
+      <c r="AL12" t="str">
+        <v>Seeweb VPC</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B13" t="str">
+        <v>99,9%</v>
+      </c>
+      <c r="C13" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D13" t="str">
+        <v>APPLICATION</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Full IaaS</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Seeweb S.r.l. - W3Suite Backend</v>
+      </c>
+      <c r="I13" t="str">
+        <v>App (RunTime) - Linux native</v>
+      </c>
+      <c r="J13" t="str">
+        <v>1 VPC</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Cloud-Single-zone</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Resources - SW configuration</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Active</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Ops Manual</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+      </c>
+      <c r="P13" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>Ops - Automated</v>
+      </c>
+      <c r="R13" t="str">
+        <v xml:space="preserve">Ops Automated (SW) - DevOps </v>
+      </c>
+      <c r="S13" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="T13" t="str">
+        <v>Configuration File (YAML)</v>
+      </c>
+      <c r="U13" t="str">
+        <v>W3 Git</v>
+      </c>
+      <c r="V13" t="str">
+        <v>SW Bins</v>
+      </c>
+      <c r="W13" t="str">
+        <v>Object Store (SW bins)</v>
+      </c>
+      <c r="X13" t="str">
+        <v>Resource Recovery</v>
+      </c>
+      <c r="Y13" t="str">
+        <v>On-Premise SW/Appliance</v>
+      </c>
+      <c r="Z13" t="str">
+        <v>On-premise Store (Appliance)</v>
+      </c>
+      <c r="AA13" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="AB13" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC13" t="str">
+        <v>1 min</v>
+      </c>
+      <c r="AD13" t="str">
+        <v>1 week</v>
+      </c>
+      <c r="AE13" t="str">
+        <v xml:space="preserve">Region Resilent </v>
+      </c>
+      <c r="AF13" t="str">
+        <v>Automated By App</v>
+      </c>
+      <c r="AG13" t="str">
+        <v>Minutes (1-5)</v>
+      </c>
+      <c r="AH13" t="str">
+        <v xml:space="preserve">Seconds </v>
+      </c>
+      <c r="AI13" t="str">
+        <v>SW Integrator</v>
+      </c>
+      <c r="AJ13" t="str">
+        <v>Deploy, API, AI Gateway, Redis Cache</v>
+      </c>
+      <c r="AK13" t="str">
+        <v>Public Cloud Consumption</v>
+      </c>
+      <c r="AL13" t="str">
+        <v>Seeweb VPC</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B14" t="str">
+        <v>99,9%</v>
+      </c>
+      <c r="C14" t="str">
+        <v>HA+</v>
+      </c>
+      <c r="D14" t="str">
+        <v>DATABASE</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Full IaaS</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Seeweb S.r.l. - PostgreSQL Primary</v>
+      </c>
+      <c r="I14" t="str">
+        <v>App (RunTime) - Linux native</v>
+      </c>
+      <c r="J14" t="str">
+        <v>1 VPC</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Cloud-Single-zone</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Resources - SW configuration</v>
+      </c>
+      <c r="M14" t="str">
+        <v xml:space="preserve">Active+ </v>
+      </c>
+      <c r="N14" t="str">
+        <v>Ops Manual</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Minutes (1-10)</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>Ops - Manual</v>
+      </c>
+      <c r="R14" t="str">
+        <v>Ops Manual - direct Log-on resource</v>
+      </c>
+      <c r="S14" t="str">
+        <v>Minutes (1-10)</v>
+      </c>
+      <c r="T14" t="str">
+        <v>Configuration File (TXT)</v>
+      </c>
+      <c r="U14" t="str">
+        <v>Vendor Versioning</v>
+      </c>
+      <c r="V14" t="str">
+        <v>SW Bins</v>
+      </c>
+      <c r="W14" t="str">
+        <v>Object Store (SW bins)</v>
+      </c>
+      <c r="X14" t="str">
+        <v>Resource: Release and Recovery</v>
+      </c>
+      <c r="Y14" t="str">
+        <v>On-Premise SW/Appliance</v>
+      </c>
+      <c r="Z14" t="str">
+        <v>On-premise Store (Appliance)</v>
+      </c>
+      <c r="AA14" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="AB14" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC14" t="str">
+        <v>1 min</v>
+      </c>
+      <c r="AD14" t="str">
+        <v>1 week</v>
+      </c>
+      <c r="AE14" t="str">
+        <v xml:space="preserve">Region Resilent </v>
+      </c>
+      <c r="AF14" t="str">
+        <v>Automated By App</v>
+      </c>
+      <c r="AG14" t="str">
+        <v>Minutes (1-5)</v>
+      </c>
+      <c r="AH14" t="str">
+        <v xml:space="preserve">Seconds </v>
+      </c>
+      <c r="AI14" t="str">
+        <v>SW Integrator</v>
+      </c>
+      <c r="AJ14" t="str">
+        <v>Backup, Tuning, PITR, WAL Shipping</v>
+      </c>
+      <c r="AK14" t="str">
+        <v>Public Cloud Consumption</v>
+      </c>
+      <c r="AL14" t="str">
+        <v>Seeweb VPC</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B15" t="str">
+        <v>99,9%</v>
+      </c>
+      <c r="C15" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D15" t="str">
+        <v>DATABASE</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Not W3 Private datacenter</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Vendor Private</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Full IaaS</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Seeweb S.r.l. - PostgreSQL Replica</v>
+      </c>
+      <c r="I15" t="str">
+        <v>App (RunTime) - Linux native</v>
+      </c>
+      <c r="J15" t="str">
+        <v>1 VPC</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Cloud-Single-zone</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Resources - SW configuration</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Standby</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Ops Manual</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
+      </c>
+      <c r="P15" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>Ops - Manual</v>
+      </c>
+      <c r="R15" t="str">
+        <v>Ops Manual - direct Log-on resource</v>
+      </c>
+      <c r="S15" t="str">
+        <v>No outages</v>
+      </c>
+      <c r="T15" t="str">
+        <v>Configuration File (TXT)</v>
+      </c>
+      <c r="U15" t="str">
+        <v>Vendor Versioning</v>
+      </c>
+      <c r="V15" t="str">
+        <v>SW Bins</v>
+      </c>
+      <c r="W15" t="str">
+        <v>Object Store (SW bins)</v>
+      </c>
+      <c r="X15" t="str">
+        <v>Resource Recovery</v>
+      </c>
+      <c r="Y15" t="str">
+        <v>On-Premise SW/Appliance</v>
+      </c>
+      <c r="Z15" t="str">
+        <v>On-premise Store (Appliance)</v>
+      </c>
+      <c r="AA15" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="AB15" t="str">
+        <v>1 month</v>
+      </c>
+      <c r="AC15" t="str">
+        <v>1 min</v>
+      </c>
+      <c r="AD15" t="str">
+        <v>1 week</v>
+      </c>
+      <c r="AE15" t="str">
+        <v xml:space="preserve">Region Resilent </v>
+      </c>
+      <c r="AF15" t="str">
+        <v>Automated By App</v>
+      </c>
+      <c r="AG15" t="str">
+        <v xml:space="preserve">Seconds </v>
+      </c>
+      <c r="AH15" t="str">
+        <v xml:space="preserve">Seconds </v>
+      </c>
+      <c r="AI15" t="str">
+        <v>SW Integrator</v>
+      </c>
+      <c r="AJ15" t="str">
+        <v>Streaming Replication, Failover Ready</v>
+      </c>
+      <c r="AK15" t="str">
+        <v>Public Cloud Consumption</v>
+      </c>
+      <c r="AL15" t="str">
+        <v>Seeweb VPC</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:AL15"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A2:G17"/>
+  <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="22.83203125" customWidth="1"/>
@@ -5788,1198 +6957,11 @@
     <col min="8" max="8" width="22.83203125" customWidth="1"/>
     <col min="9" max="9" width="22.83203125" customWidth="1"/>
     <col min="10" max="10" width="22.83203125" customWidth="1"/>
-    <col min="11" max="11" width="22.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="22.83203125" customWidth="1"/>
-    <col min="14" max="14" width="22.83203125" customWidth="1"/>
-    <col min="15" max="15" width="22.83203125" customWidth="1"/>
-    <col min="16" max="16" width="22.83203125" customWidth="1"/>
-    <col min="17" max="17" width="22.83203125" customWidth="1"/>
-    <col min="18" max="18" width="22.83203125" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" customWidth="1"/>
-    <col min="20" max="20" width="22.83203125" customWidth="1"/>
-    <col min="21" max="21" width="22.83203125" customWidth="1"/>
-    <col min="22" max="22" width="22.83203125" customWidth="1"/>
-    <col min="23" max="23" width="22.83203125" customWidth="1"/>
-    <col min="24" max="24" width="22.83203125" customWidth="1"/>
-    <col min="25" max="25" width="22.83203125" customWidth="1"/>
-    <col min="26" max="26" width="22.83203125" customWidth="1"/>
-    <col min="27" max="27" width="22.83203125" customWidth="1"/>
-    <col min="28" max="28" width="22.83203125" customWidth="1"/>
-    <col min="29" max="29" width="22.83203125" customWidth="1"/>
-    <col min="30" max="30" width="22.83203125" customWidth="1"/>
-    <col min="31" max="31" width="22.83203125" customWidth="1"/>
-    <col min="32" max="32" width="22.83203125" customWidth="1"/>
-    <col min="33" max="33" width="22.83203125" customWidth="1"/>
-    <col min="34" max="34" width="22.83203125" customWidth="1"/>
-    <col min="35" max="35" width="22.83203125" customWidth="1"/>
-    <col min="36" max="36" width="22.83203125" customWidth="1"/>
-    <col min="37" max="37" width="22.83203125" customWidth="1"/>
-    <col min="38" max="38" width="22.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>HERE YOU CAN FIND SOME NOTES TO HELP YOU UNDERSTAND HOW TO FILL IN THIS FORM. YOU CAN FIND THE COMPLETE VALUES LIST AND RELATED DESCRIPTION ON TAB "Values&amp;Description"</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Environment</v>
-      </c>
-      <c r="B5" t="str">
-        <v>SLA Model &amp; Resource Model</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
-      <c r="L5" t="str">
-        <v/>
-      </c>
-      <c r="M5" t="str">
-        <v/>
-      </c>
-      <c r="N5" t="str">
-        <v>Capacity  Model</v>
-      </c>
-      <c r="O5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-      <c r="B7" t="str">
-        <v xml:space="preserve">SLA </v>
-      </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v>Resource Model</v>
-      </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v>Resource Distribution Model &amp; HA</v>
-      </c>
-      <c r="K7" t="str">
-        <v/>
-      </c>
-      <c r="L7" t="str">
-        <v/>
-      </c>
-      <c r="M7" t="str">
-        <v/>
-      </c>
-      <c r="N7" t="str">
-        <v>Capacity Model</v>
-      </c>
-      <c r="O7" t="str">
-        <v/>
-      </c>
-      <c r="P7" t="str">
-        <v/>
-      </c>
-      <c r="Q7" t="str">
-        <v>Release Method</v>
-      </c>
-      <c r="R7" t="str">
-        <v/>
-      </c>
-      <c r="S7" t="str">
-        <v/>
-      </c>
-      <c r="T7" t="str">
-        <v>Release Configuration  &amp; Artifacts</v>
-      </c>
-      <c r="U7" t="str">
-        <v/>
-      </c>
-      <c r="V7" t="str">
-        <v/>
-      </c>
-      <c r="W7" t="str">
-        <v/>
-      </c>
-      <c r="X7" t="str">
-        <v>Use for and Method &amp; store</v>
-      </c>
-      <c r="Y7" t="str">
-        <v/>
-      </c>
-      <c r="Z7" t="str">
-        <v/>
-      </c>
-      <c r="AA7" t="str">
-        <v>Full</v>
-      </c>
-      <c r="AB7" t="str">
-        <v/>
-      </c>
-      <c r="AC7" t="str">
-        <v>Incremental (log)</v>
-      </c>
-      <c r="AD7" t="str">
-        <v/>
-      </c>
-      <c r="AE7" t="str">
-        <v>Fail-over/Fail-Back (recover full capacity)</v>
-      </c>
-      <c r="AF7" t="str">
-        <v/>
-      </c>
-      <c r="AG7" t="str">
-        <v/>
-      </c>
-      <c r="AH7" t="str">
-        <v/>
-      </c>
-      <c r="AI7" t="str">
-        <v>Operation Model</v>
-      </c>
-      <c r="AJ7" t="str">
-        <v/>
-      </c>
-      <c r="AK7" t="str">
-        <v>Cost Model</v>
-      </c>
-      <c r="AL7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str">
-        <v>ENV</v>
-      </c>
-      <c r="B8" t="str" xml:space="preserve">
-        <v xml:space="preserve">SLA
-Value</v>
-      </c>
-      <c r="C8" t="str" xml:space="preserve">
-        <v xml:space="preserve">SLA
-Class</v>
-      </c>
-      <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Proposal
- Modules</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Hosting Model</v>
-      </c>
-      <c r="F8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Hosting 
-Provider</v>
-      </c>
-      <c r="G8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Technical Model
-Module</v>
-      </c>
-      <c r="H8" t="str" xml:space="preserve">
-        <v xml:space="preserve"> Service  Resource 
-Vendor Name (Relations)</v>
-      </c>
-      <c r="I8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Service Resources 
-Implementation</v>
-      </c>
-      <c r="J8" t="str">
-        <v># instances</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Region/Zone Distribution</v>
-      </c>
-      <c r="L8" t="str">
-        <v>Distribution Method</v>
-      </c>
-      <c r="M8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Resource Role
-Distribution</v>
-      </c>
-      <c r="N8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Capacity
-Class</v>
-      </c>
-      <c r="O8" t="str">
-        <v>Method</v>
-      </c>
-      <c r="P8" t="str">
-        <v>Outages</v>
-      </c>
-      <c r="Q8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Release
-Class</v>
-      </c>
-      <c r="R8" t="str">
-        <v>Method</v>
-      </c>
-      <c r="S8" t="str">
-        <v>Outages</v>
-      </c>
-      <c r="T8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Configuration
-Specification</v>
-      </c>
-      <c r="U8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Configuration
-Version</v>
-      </c>
-      <c r="V8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Deploy
-Artifact
-</v>
-      </c>
-      <c r="W8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Artifact 
-Registry</v>
-      </c>
-      <c r="X8" t="str">
-        <v>Use for</v>
-      </c>
-      <c r="Y8" t="str">
-        <v>Method</v>
-      </c>
-      <c r="Z8" t="str">
-        <v>Store</v>
-      </c>
-      <c r="AA8" t="str">
-        <v>Freq.</v>
-      </c>
-      <c r="AB8" t="str">
-        <v>Retention</v>
-      </c>
-      <c r="AC8" t="str">
-        <v>Freq.</v>
-      </c>
-      <c r="AD8" t="str">
-        <v>Retention</v>
-      </c>
-      <c r="AE8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Recovery 
-Class</v>
-      </c>
-      <c r="AF8" t="str">
-        <v>Method</v>
-      </c>
-      <c r="AG8" t="str">
-        <v>RTO</v>
-      </c>
-      <c r="AH8" t="str">
-        <v>RPO</v>
-      </c>
-      <c r="AI8" t="str">
-        <v>Operated By</v>
-      </c>
-      <c r="AJ8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Operation other Activities
-(which  W3 activities)</v>
-      </c>
-      <c r="AK8" t="str">
-        <v>Model</v>
-      </c>
-      <c r="AL8" t="str">
-        <v>Details</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B9" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C9" t="str">
-        <v>HA</v>
-      </c>
-      <c r="D9" t="str">
-        <v>INFRASTRUCTURE</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H9" t="str">
-        <v>Seeweb S.r.l. - Proxmox VE Cluster</v>
-      </c>
-      <c r="I9" t="str">
-        <v>Virtualization Platform - ProxMox</v>
-      </c>
-      <c r="J9">
-        <v>1</v>
-      </c>
-      <c r="K9" t="str">
-        <v>Cloud-Single-zone</v>
-      </c>
-      <c r="L9" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M9" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N9" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O9" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P9" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q9" t="str">
-        <v>Ops - Manual</v>
-      </c>
-      <c r="R9" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S9" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T9" t="str">
-        <v>Configuration File (TXT)</v>
-      </c>
-      <c r="U9" t="str">
-        <v>Vendor Versioning</v>
-      </c>
-      <c r="V9" t="str">
-        <v>VMI (Virtual Machine Image) - KVM</v>
-      </c>
-      <c r="W9" t="str">
-        <v>Private Others Registry</v>
-      </c>
-      <c r="X9" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y9" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z9" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA9" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB9" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC9" t="str">
-        <v>1 min</v>
-      </c>
-      <c r="AD9" t="str">
-        <v>1 week</v>
-      </c>
-      <c r="AE9" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF9" t="str">
-        <v>Automated By App</v>
-      </c>
-      <c r="AG9" t="str">
-        <v>Minutes (1-5)</v>
-      </c>
-      <c r="AH9" t="str">
-        <v>Minutes (1-5)</v>
-      </c>
-      <c r="AI9" t="str">
-        <v>HW/SW vendor</v>
-      </c>
-      <c r="AJ9" t="str">
-        <v>Cluster Management, VM Provisioning</v>
-      </c>
-      <c r="AK9" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL9" t="str">
-        <v>Seeweb Multinodo Contract</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B10" t="str">
-        <v>99,5%</v>
-      </c>
-      <c r="C10" t="str">
-        <v>HA-</v>
-      </c>
-      <c r="D10" t="str">
-        <v>INFRASTRUCTURE</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G10" t="str">
-        <v>HW Appliance</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Seeweb S.r.l. - Fortinet FortiGate</v>
-      </c>
-      <c r="I10" t="str">
-        <v>HW Appliance - FortiGate NGFW</v>
-      </c>
-      <c r="J10">
-        <v>1</v>
-      </c>
-      <c r="K10" t="str">
-        <v>Cloud-Single-zone</v>
-      </c>
-      <c r="L10" t="str">
-        <v>Resource - Manual Installation</v>
-      </c>
-      <c r="M10" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N10" t="str">
-        <v>Fixed capacity</v>
-      </c>
-      <c r="O10" t="str">
-        <v>Do not scale - Fixed capacity</v>
-      </c>
-      <c r="P10" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q10" t="str">
-        <v>Ops - Manual</v>
-      </c>
-      <c r="R10" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S10" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T10" t="str">
-        <v>Configuration File (TXT)</v>
-      </c>
-      <c r="U10" t="str">
-        <v>Vendor Versioning</v>
-      </c>
-      <c r="V10" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W10" t="str">
-        <v>Private Others Registry</v>
-      </c>
-      <c r="X10" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y10" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z10" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA10" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB10" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC10" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AD10" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AE10" t="str">
-        <v xml:space="preserve">Local Resilent </v>
-      </c>
-      <c r="AF10" t="str">
-        <v>Manual By Operation</v>
-      </c>
-      <c r="AG10" t="str">
-        <v>Hour (1-5)</v>
-      </c>
-      <c r="AH10" t="str">
-        <v>Hour (1-5)</v>
-      </c>
-      <c r="AI10" t="str">
-        <v>HW/SW vendor</v>
-      </c>
-      <c r="AJ10" t="str">
-        <v>Security Policy, Threat Monitoring</v>
-      </c>
-      <c r="AK10" t="str">
-        <v>COTs SW License</v>
-      </c>
-      <c r="AL10" t="str">
-        <v>FortiCare via Seeweb</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B11" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C11" t="str">
-        <v>HA</v>
-      </c>
-      <c r="D11" t="str">
-        <v>INFRASTRUCTURE</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Bare Metal</v>
-      </c>
-      <c r="H11" t="str">
-        <v>Seeweb S.r.l. - Proxmox Backup Server</v>
-      </c>
-      <c r="I11" t="str">
-        <v>Bare Metal - PBS Dedicated</v>
-      </c>
-      <c r="J11">
-        <v>1</v>
-      </c>
-      <c r="K11" t="str">
-        <v>Cloud-Single-zone</v>
-      </c>
-      <c r="L11" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M11" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N11" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O11" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P11" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q11" t="str">
-        <v>Ops - Manual</v>
-      </c>
-      <c r="R11" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S11" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T11" t="str">
-        <v>Configuration File (TXT)</v>
-      </c>
-      <c r="U11" t="str">
-        <v>Vendor Versioning</v>
-      </c>
-      <c r="V11" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W11" t="str">
-        <v>Object Store (SW bins)</v>
-      </c>
-      <c r="X11" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y11" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z11" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA11" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB11" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC11" t="str">
-        <v>1 min</v>
-      </c>
-      <c r="AD11" t="str">
-        <v>1 week</v>
-      </c>
-      <c r="AE11" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF11" t="str">
-        <v>Manual By Operation</v>
-      </c>
-      <c r="AG11" t="str">
-        <v>Hour (1-5)</v>
-      </c>
-      <c r="AH11" t="str">
-        <v>Minutes (1-5)</v>
-      </c>
-      <c r="AI11" t="str">
-        <v>HW/SW vendor</v>
-      </c>
-      <c r="AJ11" t="str">
-        <v>Backup Storage, DR Recovery</v>
-      </c>
-      <c r="AK11" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL11" t="str">
-        <v>Seeweb PBS Service</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B12" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C12" t="str">
-        <v>HA</v>
-      </c>
-      <c r="D12" t="str">
-        <v>APPLICATION</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H12" t="str">
-        <v>Seeweb S.r.l. - W3Suite Frontend</v>
-      </c>
-      <c r="I12" t="str">
-        <v>App (RunTime) - Linux native</v>
-      </c>
-      <c r="J12">
-        <v>1</v>
-      </c>
-      <c r="K12" t="str">
-        <v>Cloud-Single-zone</v>
-      </c>
-      <c r="L12" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M12" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N12" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O12" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P12" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q12" t="str">
-        <v>Ops - Automated</v>
-      </c>
-      <c r="R12" t="str">
-        <v xml:space="preserve">Ops Automated (SW) - DevOps </v>
-      </c>
-      <c r="S12" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T12" t="str">
-        <v>Configuration File (YAML)</v>
-      </c>
-      <c r="U12" t="str">
-        <v>W3 Git</v>
-      </c>
-      <c r="V12" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W12" t="str">
-        <v>Object Store (SW bins)</v>
-      </c>
-      <c r="X12" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y12" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z12" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA12" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB12" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC12" t="str">
-        <v>1 min</v>
-      </c>
-      <c r="AD12" t="str">
-        <v>1 week</v>
-      </c>
-      <c r="AE12" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF12" t="str">
-        <v>Automated By App</v>
-      </c>
-      <c r="AG12" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AH12" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AI12" t="str">
-        <v>SW Integrator</v>
-      </c>
-      <c r="AJ12" t="str">
-        <v>TLS, Routing, LB Config</v>
-      </c>
-      <c r="AK12" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL12" t="str">
-        <v>Seeweb VPC</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B13" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C13" t="str">
-        <v>HA</v>
-      </c>
-      <c r="D13" t="str">
-        <v>APPLICATION</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H13" t="str">
-        <v>Seeweb S.r.l. - W3Suite Backend</v>
-      </c>
-      <c r="I13" t="str">
-        <v>App (RunTime) - Linux native</v>
-      </c>
-      <c r="J13">
-        <v>1</v>
-      </c>
-      <c r="K13" t="str">
-        <v>Cloud-Single-zone</v>
-      </c>
-      <c r="L13" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M13" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N13" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O13" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P13" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q13" t="str">
-        <v>Ops - Automated</v>
-      </c>
-      <c r="R13" t="str">
-        <v xml:space="preserve">Ops Automated (SW) - DevOps </v>
-      </c>
-      <c r="S13" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T13" t="str">
-        <v>Configuration File (YAML)</v>
-      </c>
-      <c r="U13" t="str">
-        <v>W3 Git</v>
-      </c>
-      <c r="V13" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W13" t="str">
-        <v>Object Store (SW bins)</v>
-      </c>
-      <c r="X13" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y13" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z13" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA13" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB13" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC13" t="str">
-        <v>1 min</v>
-      </c>
-      <c r="AD13" t="str">
-        <v>1 week</v>
-      </c>
-      <c r="AE13" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF13" t="str">
-        <v>Automated By App</v>
-      </c>
-      <c r="AG13" t="str">
-        <v>Minutes (1-5)</v>
-      </c>
-      <c r="AH13" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AI13" t="str">
-        <v>SW Integrator</v>
-      </c>
-      <c r="AJ13" t="str">
-        <v>Deploy, API, AI Gateway, Cache</v>
-      </c>
-      <c r="AK13" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL13" t="str">
-        <v>Seeweb VPC</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B14" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C14" t="str">
-        <v>HA+</v>
-      </c>
-      <c r="D14" t="str">
-        <v>DATABASE</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H14" t="str">
-        <v>Seeweb S.r.l. - PostgreSQL Primary</v>
-      </c>
-      <c r="I14" t="str">
-        <v>App (RunTime) - Linux native</v>
-      </c>
-      <c r="J14">
-        <v>1</v>
-      </c>
-      <c r="K14" t="str">
-        <v>Cloud-Single-zone</v>
-      </c>
-      <c r="L14" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M14" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N14" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O14" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P14" t="str">
-        <v>Minutes (1-10)</v>
-      </c>
-      <c r="Q14" t="str">
-        <v>Ops - Manual</v>
-      </c>
-      <c r="R14" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S14" t="str">
-        <v>Minutes (1-10)</v>
-      </c>
-      <c r="T14" t="str">
-        <v>Configuration File (TXT)</v>
-      </c>
-      <c r="U14" t="str">
-        <v>Vendor Versioning</v>
-      </c>
-      <c r="V14" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W14" t="str">
-        <v>Object Store (SW bins)</v>
-      </c>
-      <c r="X14" t="str">
-        <v>Resource: Release and Recovery</v>
-      </c>
-      <c r="Y14" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z14" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA14" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB14" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC14" t="str">
-        <v>1 min</v>
-      </c>
-      <c r="AD14" t="str">
-        <v>1 week</v>
-      </c>
-      <c r="AE14" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF14" t="str">
-        <v>Automated By App</v>
-      </c>
-      <c r="AG14" t="str">
-        <v>Minutes (1-5)</v>
-      </c>
-      <c r="AH14" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AI14" t="str">
-        <v>SW Integrator</v>
-      </c>
-      <c r="AJ14" t="str">
-        <v>Backup, Tuning, PITR, WAL</v>
-      </c>
-      <c r="AK14" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL14" t="str">
-        <v>Seeweb VPC</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>PROD</v>
-      </c>
-      <c r="B15" t="str">
-        <v>99,9%</v>
-      </c>
-      <c r="C15" t="str">
-        <v>HA</v>
-      </c>
-      <c r="D15" t="str">
-        <v>DATABASE</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Not W3 Private datacenter</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Vendor Private</v>
-      </c>
-      <c r="G15" t="str">
-        <v>Full IaaS</v>
-      </c>
-      <c r="H15" t="str">
-        <v>Seeweb S.r.l. - PostgreSQL Replica</v>
-      </c>
-      <c r="I15" t="str">
-        <v>App (RunTime) - Linux native</v>
-      </c>
-      <c r="J15">
-        <v>1</v>
-      </c>
-      <c r="K15" t="str">
-        <v>Cloud-Single-zone</v>
-      </c>
-      <c r="L15" t="str">
-        <v>Resources - SW configuration</v>
-      </c>
-      <c r="M15" t="str">
-        <v>Standby</v>
-      </c>
-      <c r="N15" t="str">
-        <v>Ops Manual</v>
-      </c>
-      <c r="O15" t="str">
-        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
-      </c>
-      <c r="P15" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="Q15" t="str">
-        <v>Ops - Manual</v>
-      </c>
-      <c r="R15" t="str">
-        <v>Ops Manual - direct Log-on resource</v>
-      </c>
-      <c r="S15" t="str">
-        <v>No outages</v>
-      </c>
-      <c r="T15" t="str">
-        <v>Configuration File (TXT)</v>
-      </c>
-      <c r="U15" t="str">
-        <v>Vendor Versioning</v>
-      </c>
-      <c r="V15" t="str">
-        <v>SW Bins</v>
-      </c>
-      <c r="W15" t="str">
-        <v>Object Store (SW bins)</v>
-      </c>
-      <c r="X15" t="str">
-        <v>Resource Recovery</v>
-      </c>
-      <c r="Y15" t="str">
-        <v>On-Premise SW/Appliance</v>
-      </c>
-      <c r="Z15" t="str">
-        <v>On-premise Store (Appliance)</v>
-      </c>
-      <c r="AA15" t="str">
-        <v>Daily</v>
-      </c>
-      <c r="AB15" t="str">
-        <v>1 month</v>
-      </c>
-      <c r="AC15" t="str">
-        <v>1 min</v>
-      </c>
-      <c r="AD15" t="str">
-        <v>1 week</v>
-      </c>
-      <c r="AE15" t="str">
-        <v xml:space="preserve">Region Resilent </v>
-      </c>
-      <c r="AF15" t="str">
-        <v>Automated By App</v>
-      </c>
-      <c r="AG15" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AH15" t="str">
-        <v xml:space="preserve">Seconds </v>
-      </c>
-      <c r="AI15" t="str">
-        <v>SW Integrator</v>
-      </c>
-      <c r="AJ15" t="str">
-        <v>Streaming Replication, Failover</v>
-      </c>
-      <c r="AK15" t="str">
-        <v>Public Cloud Consumption</v>
-      </c>
-      <c r="AL15" t="str">
-        <v>Seeweb VPC</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AL15"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:G15"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-    <col min="6" max="6" width="25.83203125" customWidth="1"/>
-    <col min="7" max="7" width="25.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-    <col min="9" max="9" width="25.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="A2" t="str">
-        <v>Public Cloud Zones or W3 Sites</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Field Definition &amp; Values 
-Module of solution</v>
-      </c>
-      <c r="B3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Field Definition &amp; Values 
-Resource of module</v>
-      </c>
-      <c r="C3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Field Definition &amp; Values
-Resource component</v>
-      </c>
-      <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Field Definition &amp; Values
-Sites List</v>
+        <v>Public Cloud Zones or W3 Sites - Seeweb Italy</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -6992,19 +6974,21 @@
       </c>
       <c r="C7" t="str" xml:space="preserve">
         <v xml:space="preserve">Resource 
-Component (if needed)</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Region (Zone/site)</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Zone/site</v>
+Component</v>
+      </c>
+      <c r="D7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Seeweb DC1
+(Primary)</v>
+      </c>
+      <c r="E7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Seeweb DC2
+(DR)</v>
       </c>
       <c r="F7" t="str">
-        <v>Zone/site</v>
+        <v>Seeweb DC3</v>
       </c>
       <c r="G7" t="str">
-        <v>Zone/site</v>
+        <v>Notes</v>
       </c>
     </row>
     <row r="8">
@@ -7018,10 +7002,10 @@
         <v/>
       </c>
       <c r="D8" t="str">
-        <v>Seeweb Italy DC1</v>
+        <v>Milan/Rome</v>
       </c>
       <c r="E8" t="str">
-        <v>Seeweb Italy DC2</v>
+        <v>Rome/Milan</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -7038,10 +7022,10 @@
         <v>Proxmox VE Cluster</v>
       </c>
       <c r="C9" t="str">
-        <v>Multinodo Cluster</v>
+        <v>Nodo 1</v>
       </c>
       <c r="D9" t="str">
-        <v>Seeweb DC1 (Primary)</v>
+        <v>Active</v>
       </c>
       <c r="E9" t="str">
         <v/>
@@ -7050,7 +7034,7 @@
         <v/>
       </c>
       <c r="G9" t="str">
-        <v/>
+        <v>Primary compute</v>
       </c>
     </row>
     <row r="10">
@@ -7058,13 +7042,13 @@
         <v>INFRASTRUCTURE</v>
       </c>
       <c r="B10" t="str">
-        <v>FortiGate NGFW</v>
+        <v>Proxmox VE Cluster</v>
       </c>
       <c r="C10" t="str">
-        <v>Single Appliance</v>
+        <v>Nodo 2</v>
       </c>
       <c r="D10" t="str">
-        <v>Seeweb DC1</v>
+        <v>Active</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -7073,7 +7057,7 @@
         <v/>
       </c>
       <c r="G10" t="str">
-        <v/>
+        <v>HA compute</v>
       </c>
     </row>
     <row r="11">
@@ -7081,36 +7065,36 @@
         <v>INFRASTRUCTURE</v>
       </c>
       <c r="B11" t="str">
-        <v>Proxmox Backup Server</v>
+        <v>Proxmox VE Cluster</v>
       </c>
       <c r="C11" t="str">
-        <v>Dedicated Server</v>
+        <v>Nodo 3</v>
       </c>
       <c r="D11" t="str">
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Seeweb DC2 (DR)</v>
+        <v>Active</v>
       </c>
       <c r="F11" t="str">
         <v/>
       </c>
       <c r="G11" t="str">
-        <v/>
+        <v>DR compute</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>APPLICATION</v>
+        <v>INFRASTRUCTURE</v>
       </c>
       <c r="B12" t="str">
-        <v>W3Suite Frontend</v>
+        <v>FortiGate NGFW</v>
       </c>
       <c r="C12" t="str">
-        <v>Nginx + LB</v>
+        <v>Single Appliance</v>
       </c>
       <c r="D12" t="str">
-        <v>Seeweb DC1</v>
+        <v>Active</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -7119,44 +7103,44 @@
         <v/>
       </c>
       <c r="G12" t="str">
-        <v/>
+        <v>HW Appliance - No HA</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>APPLICATION</v>
+        <v>INFRASTRUCTURE</v>
       </c>
       <c r="B13" t="str">
-        <v>W3Suite Backend</v>
+        <v>Proxmox Backup Server</v>
       </c>
       <c r="C13" t="str">
-        <v>API + Redis + MCP</v>
+        <v>Dedicated</v>
       </c>
       <c r="D13" t="str">
-        <v>Seeweb DC1</v>
+        <v/>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>Active</v>
       </c>
       <c r="F13" t="str">
         <v/>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>DR Backup Storage</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>DATABASE</v>
+        <v>APPLICATION</v>
       </c>
       <c r="B14" t="str">
-        <v>PostgreSQL Primary</v>
+        <v>W3Suite Frontend</v>
       </c>
       <c r="C14" t="str">
-        <v>DB Primary</v>
+        <v>Nginx + LB</v>
       </c>
       <c r="D14" t="str">
-        <v>Seeweb DC1</v>
+        <v>Active</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -7170,16 +7154,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>DATABASE</v>
+        <v>APPLICATION</v>
       </c>
       <c r="B15" t="str">
-        <v>PostgreSQL Replica</v>
+        <v>W3Suite Backend</v>
       </c>
       <c r="C15" t="str">
-        <v>DB Standby</v>
+        <v>API + Redis + MCP</v>
       </c>
       <c r="D15" t="str">
-        <v>Seeweb DC1</v>
+        <v>Active</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -7191,9 +7175,55 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>DATABASE</v>
+      </c>
+      <c r="B16" t="str">
+        <v>PostgreSQL Primary</v>
+      </c>
+      <c r="C16" t="str">
+        <v>DB Primary</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Active</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v>Read/Write</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>DATABASE</v>
+      </c>
+      <c r="B17" t="str">
+        <v>PostgreSQL Replica</v>
+      </c>
+      <c r="C17" t="str">
+        <v>DB Standby</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Standby</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v>Streaming Replication</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:G15"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:G17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update resource models for Seeweb Proxmox cluster deployments
Update the Excel file to reflect the correct technical models for Seeweb's Proxmox Backup Server (PBS) and FortiGate appliances, changing PBS from 'Bare Metal' to 'Full IaaS' and FortiGate from 'Cloud-Single-zone' to 'Full IaaS' based on Seeweb's service offerings.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: acde2c79-b7bb-415e-aca2-c6d44a8513d3
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
+++ b/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
@@ -5820,7 +5820,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>W3Suite - Service Resource Model - Seeweb Infrastructure</v>
+        <v>W3Suite - Service Resource Model - Seeweb Infrastructure (Verified)</v>
       </c>
     </row>
     <row r="4">
@@ -6144,13 +6144,13 @@
         <v>Vendor Private</v>
       </c>
       <c r="G9" t="str">
-        <v>Full IaaS</v>
+        <v>Bare Metal</v>
       </c>
       <c r="H9" t="str">
-        <v>Seeweb S.r.l. - Proxmox VE Cluster</v>
+        <v>Seeweb S.r.l. - Foundation Server Cluster</v>
       </c>
       <c r="I9" t="str">
-        <v>Virtualization Platform - ProxMox</v>
+        <v>Bare Metal - Proxmox VE Hosts</v>
       </c>
       <c r="J9" t="str">
         <v>3+ nodi</v>
@@ -6237,7 +6237,7 @@
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL9" t="str">
-        <v>Seeweb Multinodo Contract</v>
+        <v>Seeweb Foundation Server Contract</v>
       </c>
     </row>
     <row r="10">
@@ -6260,31 +6260,31 @@
         <v>Vendor Private</v>
       </c>
       <c r="G10" t="str">
-        <v>HW Appliance</v>
+        <v>Full IaaS</v>
       </c>
       <c r="H10" t="str">
-        <v>Seeweb S.r.l. - Fortinet FortiGate</v>
+        <v>Seeweb S.r.l. - Fortinet FortiGate VM</v>
       </c>
       <c r="I10" t="str">
-        <v>HW Appliance - FortiGate NGFW</v>
+        <v>Virtual Appliance - FortiGate NGFW</v>
       </c>
       <c r="J10" t="str">
         <v>1 (Single)</v>
       </c>
       <c r="K10" t="str">
-        <v>N/A</v>
+        <v>Cloud-Single-zone</v>
       </c>
       <c r="L10" t="str">
-        <v>Resource - Manual Installation</v>
+        <v>Resources - SW configuration</v>
       </c>
       <c r="M10" t="str">
         <v>Active</v>
       </c>
       <c r="N10" t="str">
-        <v>Fixed capacity</v>
+        <v>Ops Manual</v>
       </c>
       <c r="O10" t="str">
-        <v>Do not scale - Fixed capacity</v>
+        <v>Ops Manual - Cloud consolle/direct Log-on resource</v>
       </c>
       <c r="P10" t="str">
         <v>No outages</v>
@@ -6305,7 +6305,7 @@
         <v>Vendor Versioning</v>
       </c>
       <c r="V10" t="str">
-        <v>SW Bins</v>
+        <v>VMI (Virtual Machine Image) - KVM</v>
       </c>
       <c r="W10" t="str">
         <v>Private Others Registry</v>
@@ -6350,10 +6350,10 @@
         <v>Security Policy, Threat Monitoring, FW Rules</v>
       </c>
       <c r="AK10" t="str">
-        <v>(on-premise) HW Buy &amp; Support</v>
+        <v>COTs SW License</v>
       </c>
       <c r="AL10" t="str">
-        <v>FortiGate HW + FortiCare Support</v>
+        <v>FortiGate VM + FortiCare Support</v>
       </c>
     </row>
     <row r="11">
@@ -6376,16 +6376,16 @@
         <v>Vendor Private</v>
       </c>
       <c r="G11" t="str">
-        <v>Bare Metal</v>
+        <v>Full IaaS</v>
       </c>
       <c r="H11" t="str">
-        <v>Seeweb S.r.l. - Proxmox Backup Server</v>
+        <v>Seeweb S.r.l. - Cloud Backup (PBS)</v>
       </c>
       <c r="I11" t="str">
-        <v>Bare Metal - PBS Dedicated</v>
+        <v>Cloud Service - Proxmox Backup Server</v>
       </c>
       <c r="J11" t="str">
-        <v>1 (Dedicato)</v>
+        <v>1 (Servizio)</v>
       </c>
       <c r="K11" t="str">
         <v>Cloud-Single-zone</v>
@@ -6469,7 +6469,7 @@
         <v>Public Cloud Consumption</v>
       </c>
       <c r="AL11" t="str">
-        <v>Seeweb PBS Service</v>
+        <v>Seeweb Cloud Backup 23€/100GB</v>
       </c>
     </row>
     <row r="12">
@@ -6945,7 +6945,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:G17"/>
+  <dimension ref="A2:F17"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -6961,7 +6961,7 @@
   <sheetData>
     <row r="2">
       <c r="A2" t="str">
-        <v>Public Cloud Zones or W3 Sites - Seeweb Italy</v>
+        <v>Public Cloud Zones or W3 Sites - Seeweb Italy (Verified from seeweb.it)</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -6985,9 +6985,6 @@
 (DR)</v>
       </c>
       <c r="F7" t="str">
-        <v>Seeweb DC3</v>
-      </c>
-      <c r="G7" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -7002,15 +6999,12 @@
         <v/>
       </c>
       <c r="D8" t="str">
-        <v>Milan/Rome</v>
+        <v>Foundation Server</v>
       </c>
       <c r="E8" t="str">
-        <v>Rome/Milan</v>
+        <v>Cloud Backup</v>
       </c>
       <c r="F8" t="str">
-        <v/>
-      </c>
-      <c r="G8" t="str">
         <v/>
       </c>
     </row>
@@ -7019,10 +7013,10 @@
         <v>INFRASTRUCTURE</v>
       </c>
       <c r="B9" t="str">
-        <v>Proxmox VE Cluster</v>
+        <v>Foundation Server Cluster</v>
       </c>
       <c r="C9" t="str">
-        <v>Nodo 1</v>
+        <v>Nodo 1 (Bare Metal)</v>
       </c>
       <c r="D9" t="str">
         <v>Active</v>
@@ -7031,10 +7025,7 @@
         <v/>
       </c>
       <c r="F9" t="str">
-        <v/>
-      </c>
-      <c r="G9" t="str">
-        <v>Primary compute</v>
+        <v>Proxmox VE Host</v>
       </c>
     </row>
     <row r="10">
@@ -7042,10 +7033,10 @@
         <v>INFRASTRUCTURE</v>
       </c>
       <c r="B10" t="str">
-        <v>Proxmox VE Cluster</v>
+        <v>Foundation Server Cluster</v>
       </c>
       <c r="C10" t="str">
-        <v>Nodo 2</v>
+        <v>Nodo 2 (Bare Metal)</v>
       </c>
       <c r="D10" t="str">
         <v>Active</v>
@@ -7054,10 +7045,7 @@
         <v/>
       </c>
       <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10" t="str">
-        <v>HA compute</v>
+        <v>Proxmox VE Host</v>
       </c>
     </row>
     <row r="11">
@@ -7065,10 +7053,10 @@
         <v>INFRASTRUCTURE</v>
       </c>
       <c r="B11" t="str">
-        <v>Proxmox VE Cluster</v>
+        <v>Foundation Server Cluster</v>
       </c>
       <c r="C11" t="str">
-        <v>Nodo 3</v>
+        <v>Nodo 3 (Bare Metal)</v>
       </c>
       <c r="D11" t="str">
         <v/>
@@ -7077,10 +7065,7 @@
         <v>Active</v>
       </c>
       <c r="F11" t="str">
-        <v/>
-      </c>
-      <c r="G11" t="str">
-        <v>DR compute</v>
+        <v>DR Node</v>
       </c>
     </row>
     <row r="12">
@@ -7088,10 +7073,10 @@
         <v>INFRASTRUCTURE</v>
       </c>
       <c r="B12" t="str">
-        <v>FortiGate NGFW</v>
+        <v>FortiGate VM</v>
       </c>
       <c r="C12" t="str">
-        <v>Single Appliance</v>
+        <v>Virtual Appliance</v>
       </c>
       <c r="D12" t="str">
         <v>Active</v>
@@ -7100,10 +7085,7 @@
         <v/>
       </c>
       <c r="F12" t="str">
-        <v/>
-      </c>
-      <c r="G12" t="str">
-        <v>HW Appliance - No HA</v>
+        <v>NGFW (1-4 CPU)</v>
       </c>
     </row>
     <row r="13">
@@ -7111,10 +7093,10 @@
         <v>INFRASTRUCTURE</v>
       </c>
       <c r="B13" t="str">
-        <v>Proxmox Backup Server</v>
+        <v>Cloud Backup (PBS)</v>
       </c>
       <c r="C13" t="str">
-        <v>Dedicated</v>
+        <v>Cloud Service</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -7123,10 +7105,7 @@
         <v>Active</v>
       </c>
       <c r="F13" t="str">
-        <v/>
-      </c>
-      <c r="G13" t="str">
-        <v>DR Backup Storage</v>
+        <v>23€/100GB</v>
       </c>
     </row>
     <row r="14">
@@ -7137,7 +7116,7 @@
         <v>W3Suite Frontend</v>
       </c>
       <c r="C14" t="str">
-        <v>Nginx + LB</v>
+        <v>VPC (VM)</v>
       </c>
       <c r="D14" t="str">
         <v>Active</v>
@@ -7146,10 +7125,7 @@
         <v/>
       </c>
       <c r="F14" t="str">
-        <v/>
-      </c>
-      <c r="G14" t="str">
-        <v/>
+        <v>Nginx + LB</v>
       </c>
     </row>
     <row r="15">
@@ -7160,7 +7136,7 @@
         <v>W3Suite Backend</v>
       </c>
       <c r="C15" t="str">
-        <v>API + Redis + MCP</v>
+        <v>VPC (VM)</v>
       </c>
       <c r="D15" t="str">
         <v>Active</v>
@@ -7169,10 +7145,7 @@
         <v/>
       </c>
       <c r="F15" t="str">
-        <v/>
-      </c>
-      <c r="G15" t="str">
-        <v/>
+        <v>API + Redis + MCP</v>
       </c>
     </row>
     <row r="16">
@@ -7183,7 +7156,7 @@
         <v>PostgreSQL Primary</v>
       </c>
       <c r="C16" t="str">
-        <v>DB Primary</v>
+        <v>VPC (VM)</v>
       </c>
       <c r="D16" t="str">
         <v>Active</v>
@@ -7192,9 +7165,6 @@
         <v/>
       </c>
       <c r="F16" t="str">
-        <v/>
-      </c>
-      <c r="G16" t="str">
         <v>Read/Write</v>
       </c>
     </row>
@@ -7206,7 +7176,7 @@
         <v>PostgreSQL Replica</v>
       </c>
       <c r="C17" t="str">
-        <v>DB Standby</v>
+        <v>VPC (VM)</v>
       </c>
       <c r="D17" t="str">
         <v>Standby</v>
@@ -7215,15 +7185,12 @@
         <v/>
       </c>
       <c r="F17" t="str">
-        <v/>
-      </c>
-      <c r="G17" t="str">
         <v>Streaming Replication</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:G17"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update service resource distribution with a two-node cluster
Correct the service resource distribution to reflect a two-node cluster configuration for the Foundation Server and adjust the disaster recovery site accordingly.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4c6f02d1-018a-458d-8cea-a3a84f53996d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
+++ b/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
@@ -5820,7 +5820,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>W3Suite - Service Resource Model - Seeweb Infrastructure (Verified)</v>
+        <v>W3Suite - Service Resource Model - Seeweb Infrastructure</v>
       </c>
     </row>
     <row r="4">
@@ -6153,10 +6153,10 @@
         <v>Bare Metal - Proxmox VE Hosts</v>
       </c>
       <c r="J9" t="str">
-        <v>3+ nodi</v>
+        <v>2 nodi</v>
       </c>
       <c r="K9" t="str">
-        <v xml:space="preserve">Cloud-Multi-region </v>
+        <v>Cloud-Multi-zone</v>
       </c>
       <c r="L9" t="str">
         <v>Resources - SW configuration</v>
@@ -6216,7 +6216,7 @@
         <v>1 week</v>
       </c>
       <c r="AE9" t="str">
-        <v xml:space="preserve">Region Resilent </v>
+        <v xml:space="preserve">Zone Resilent </v>
       </c>
       <c r="AF9" t="str">
         <v>Automated By App</v>
@@ -6945,7 +6945,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:F17"/>
+  <dimension ref="A2:F16"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -6961,7 +6961,7 @@
   <sheetData>
     <row r="2">
       <c r="A2" t="str">
-        <v>Public Cloud Zones or W3 Sites - Seeweb Italy (Verified from seeweb.it)</v>
+        <v>Public Cloud Zones or W3 Sites - Seeweb Italy</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="E7" t="str" xml:space="preserve">
         <v xml:space="preserve">Seeweb DC2
-(DR)</v>
+(Backup)</v>
       </c>
       <c r="F7" t="str">
         <v>Notes</v>
@@ -7045,7 +7045,7 @@
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Proxmox VE Host</v>
+        <v>Proxmox VE Host + HA Appliance</v>
       </c>
     </row>
     <row r="11">
@@ -7053,19 +7053,19 @@
         <v>INFRASTRUCTURE</v>
       </c>
       <c r="B11" t="str">
-        <v>Foundation Server Cluster</v>
+        <v>FortiGate VM</v>
       </c>
       <c r="C11" t="str">
-        <v>Nodo 3 (Bare Metal)</v>
+        <v>Virtual Appliance</v>
       </c>
       <c r="D11" t="str">
+        <v>Active</v>
+      </c>
+      <c r="E11" t="str">
         <v/>
       </c>
-      <c r="E11" t="str">
-        <v>Active</v>
-      </c>
       <c r="F11" t="str">
-        <v>DR Node</v>
+        <v>NGFW (1-4 CPU)</v>
       </c>
     </row>
     <row r="12">
@@ -7073,39 +7073,39 @@
         <v>INFRASTRUCTURE</v>
       </c>
       <c r="B12" t="str">
-        <v>FortiGate VM</v>
+        <v>Cloud Backup (PBS)</v>
       </c>
       <c r="C12" t="str">
-        <v>Virtual Appliance</v>
+        <v>Cloud Service</v>
       </c>
       <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
         <v>Active</v>
       </c>
-      <c r="E12" t="str">
-        <v/>
-      </c>
       <c r="F12" t="str">
-        <v>NGFW (1-4 CPU)</v>
+        <v>23€/100GB - DR</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>INFRASTRUCTURE</v>
+        <v>APPLICATION</v>
       </c>
       <c r="B13" t="str">
-        <v>Cloud Backup (PBS)</v>
+        <v>W3Suite Frontend</v>
       </c>
       <c r="C13" t="str">
-        <v>Cloud Service</v>
+        <v>VPC (VM)</v>
       </c>
       <c r="D13" t="str">
+        <v>Active</v>
+      </c>
+      <c r="E13" t="str">
         <v/>
       </c>
-      <c r="E13" t="str">
-        <v>Active</v>
-      </c>
       <c r="F13" t="str">
-        <v>23€/100GB</v>
+        <v>Nginx + LB</v>
       </c>
     </row>
     <row r="14">
@@ -7113,7 +7113,7 @@
         <v>APPLICATION</v>
       </c>
       <c r="B14" t="str">
-        <v>W3Suite Frontend</v>
+        <v>W3Suite Backend</v>
       </c>
       <c r="C14" t="str">
         <v>VPC (VM)</v>
@@ -7125,15 +7125,15 @@
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>Nginx + LB</v>
+        <v>API + Redis + MCP</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>APPLICATION</v>
+        <v>DATABASE</v>
       </c>
       <c r="B15" t="str">
-        <v>W3Suite Backend</v>
+        <v>PostgreSQL Primary</v>
       </c>
       <c r="C15" t="str">
         <v>VPC (VM)</v>
@@ -7145,7 +7145,7 @@
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>API + Redis + MCP</v>
+        <v>Read/Write</v>
       </c>
     </row>
     <row r="16">
@@ -7153,44 +7153,24 @@
         <v>DATABASE</v>
       </c>
       <c r="B16" t="str">
-        <v>PostgreSQL Primary</v>
+        <v>PostgreSQL Replica</v>
       </c>
       <c r="C16" t="str">
         <v>VPC (VM)</v>
       </c>
       <c r="D16" t="str">
-        <v>Active</v>
+        <v>Standby</v>
       </c>
       <c r="E16" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>Read/Write</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>DATABASE</v>
-      </c>
-      <c r="B17" t="str">
-        <v>PostgreSQL Replica</v>
-      </c>
-      <c r="C17" t="str">
-        <v>VPC (VM)</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Standby</v>
-      </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
         <v>Streaming Replication</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:F17"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:F16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update backup configuration to include all machines
Update the Excel file to reflect that all virtual machines now have both snapshot and incremental backups enabled.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c04d42b7-84ea-43ca-a036-4251526c58fe
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
+++ b/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE-FINAL.xlsx
@@ -6195,7 +6195,7 @@
         <v>Private Others Registry</v>
       </c>
       <c r="X9" t="str">
-        <v>Resource Recovery</v>
+        <v>Resource: Release and Recovery</v>
       </c>
       <c r="Y9" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -6311,7 +6311,7 @@
         <v>Private Others Registry</v>
       </c>
       <c r="X10" t="str">
-        <v>Resource Recovery</v>
+        <v>Resource: Release and Recovery</v>
       </c>
       <c r="Y10" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -6326,13 +6326,13 @@
         <v>1 month</v>
       </c>
       <c r="AC10" t="str">
-        <v>N/A</v>
+        <v>1 min</v>
       </c>
       <c r="AD10" t="str">
-        <v>N/A</v>
+        <v>1 week</v>
       </c>
       <c r="AE10" t="str">
-        <v xml:space="preserve">Local Resilent </v>
+        <v xml:space="preserve">Region Resilent </v>
       </c>
       <c r="AF10" t="str">
         <v>Manual By Operation</v>
@@ -6341,7 +6341,7 @@
         <v>Hour (1-5)</v>
       </c>
       <c r="AH10" t="str">
-        <v>Hour (1-5)</v>
+        <v>Minutes (1-5)</v>
       </c>
       <c r="AI10" t="str">
         <v>HW/SW vendor</v>
@@ -6463,7 +6463,7 @@
         <v>HW/SW vendor</v>
       </c>
       <c r="AJ11" t="str">
-        <v>Backup Storage, DR Recovery, Retention</v>
+        <v>Backup Storage, Snapshot + Incremental, DR Recovery</v>
       </c>
       <c r="AK11" t="str">
         <v>Public Cloud Consumption</v>
@@ -6543,7 +6543,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X12" t="str">
-        <v>Resource Recovery</v>
+        <v>Resource: Release and Recovery</v>
       </c>
       <c r="Y12" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -6659,7 +6659,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X13" t="str">
-        <v>Resource Recovery</v>
+        <v>Resource: Release and Recovery</v>
       </c>
       <c r="Y13" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -6891,7 +6891,7 @@
         <v>Object Store (SW bins)</v>
       </c>
       <c r="X15" t="str">
-        <v>Resource Recovery</v>
+        <v>Resource: Release and Recovery</v>
       </c>
       <c r="Y15" t="str">
         <v>On-Premise SW/Appliance</v>
@@ -6945,7 +6945,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:F16"/>
+  <dimension ref="A2:G16"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -6985,6 +6985,9 @@
 (Backup)</v>
       </c>
       <c r="F7" t="str">
+        <v>Backup Type</v>
+      </c>
+      <c r="G7" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -7007,6 +7010,9 @@
       <c r="F8" t="str">
         <v/>
       </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -7025,6 +7031,9 @@
         <v/>
       </c>
       <c r="F9" t="str">
+        <v>Snapshot + Incr</v>
+      </c>
+      <c r="G9" t="str">
         <v>Proxmox VE Host</v>
       </c>
     </row>
@@ -7045,7 +7054,10 @@
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Proxmox VE Host + HA Appliance</v>
+        <v>Snapshot + Incr</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Proxmox VE Host + HA</v>
       </c>
     </row>
     <row r="11">
@@ -7065,7 +7077,10 @@
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>NGFW (1-4 CPU)</v>
+        <v>Snapshot + Incr</v>
+      </c>
+      <c r="G11" t="str">
+        <v>NGFW</v>
       </c>
     </row>
     <row r="12">
@@ -7085,7 +7100,10 @@
         <v>Active</v>
       </c>
       <c r="F12" t="str">
-        <v>23€/100GB - DR</v>
+        <v>-</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Backup Target DC2</v>
       </c>
     </row>
     <row r="13">
@@ -7105,6 +7123,9 @@
         <v/>
       </c>
       <c r="F13" t="str">
+        <v>Snapshot + Incr</v>
+      </c>
+      <c r="G13" t="str">
         <v>Nginx + LB</v>
       </c>
     </row>
@@ -7125,6 +7146,9 @@
         <v/>
       </c>
       <c r="F14" t="str">
+        <v>Snapshot + Incr</v>
+      </c>
+      <c r="G14" t="str">
         <v>API + Redis + MCP</v>
       </c>
     </row>
@@ -7145,7 +7169,10 @@
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>Read/Write</v>
+        <v>Snapshot + Incr</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Read/Write + WAL</v>
       </c>
     </row>
     <row r="16">
@@ -7165,12 +7192,15 @@
         <v/>
       </c>
       <c r="F16" t="str">
+        <v>Snapshot + Incr</v>
+      </c>
+      <c r="G16" t="str">
         <v>Streaming Replication</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:F16"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>